<commit_message>
115 ⇒ fase IV ⇒ tancament fase III de proves E2E: pilot Chrome, resume, Excel i cleanup validats
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5819" uniqueCount="816">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6491" uniqueCount="946">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -2590,6 +2590,411 @@
   </si>
   <si>
     <t>Referència revalidació</t>
+  </si>
+  <si>
+    <t>sim-20260913T111019655Z-9e0891f2</t>
+  </si>
+  <si>
+    <t>sim-20260913T111019655Z-9e0891f2--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>Blink</t>
+  </si>
+  <si>
+    <t>153.0.8010.36</t>
+  </si>
+  <si>
+    <t>LOCAL</t>
+  </si>
+  <si>
+    <t>7e9dd1522f490095168216db66eca0832f724bd0</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:19.659Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:22.141Z</t>
+  </si>
+  <si>
+    <t>PASSED</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Escenari pilot completat correctament.</t>
+  </si>
+  <si>
+    <t>SYNCED</t>
+  </si>
+  <si>
+    <t>sim-20260913T111041125Z-ed96abb8</t>
+  </si>
+  <si>
+    <t>sim-20260913T111041125Z-ed96abb8--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:41.130Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:42.751Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T111041125Z-ed96abb8--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:42.755Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:51.579Z</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">expect(locator).toBeVisible() failed
+Locator: getByRole('heading', { name: 'Encara no tens favorits.' })
+Expected: visible
+Timeout: 5000ms
+Error: element(s) not found
+Call log:
+  - Expect "to.be.visible" with timeout 5000ms
+  - waiting for getByRole('heading', { name: 'Encara no tens favorits.' })
+</t>
+  </si>
+  <si>
+    <t>/DATA/repos/zuppeto/e2e/.runs/artifacts/ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>sim-20260913T111041125Z-ed96abb8--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:51.582Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:10:54.122Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T112900902Z-2255535c</t>
+  </si>
+  <si>
+    <t>sim-20260913T112900902Z-2255535c--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:29:00.907Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:29:03.493Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: No s'ha pogut consultar els favorits E2E (404).
+    at eval (eval at evaluate (:302:30), &lt;anonymous&gt;:12:23)
+    at async &lt;anonymous&gt;:328:30</t>
+  </si>
+  <si>
+    <t>sim-20260913T112946531Z-c862bf18</t>
+  </si>
+  <si>
+    <t>sim-20260913T112946531Z-c862bf18--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:29:46.536Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:29:50.909Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T113026780Z-8339bf7a</t>
+  </si>
+  <si>
+    <t>sim-20260913T113026780Z-8339bf7a--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:30:26.785Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:30:32.278Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T113124470Z-5156e994</t>
+  </si>
+  <si>
+    <t>sim-20260913T113124470Z-5156e994--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:31:24.482Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:31:32.020Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T113438964Z-c4d2add2</t>
+  </si>
+  <si>
+    <t>sim-20260913T113438964Z-c4d2add2--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:34:38.973Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:34:52.945Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T113523799Z-8419242a</t>
+  </si>
+  <si>
+    <t>sim-20260913T113523799Z-8419242a--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:35:23.829Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:35:37.057Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T113601623Z-b4c32d17</t>
+  </si>
+  <si>
+    <t>sim-20260913T113601623Z-b4c32d17--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:36:01.630Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:36:13.449Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T113644644Z-c9cfd57d</t>
+  </si>
+  <si>
+    <t>sim-20260913T113644644Z-c9cfd57d--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:36:44.659Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:36:57.492Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114139652Z-99b9a8c3</t>
+  </si>
+  <si>
+    <t>sim-20260913T114139652Z-99b9a8c3--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:41:39.689Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:41:46.087Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114139652Z-99b9a8c3--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:41:46.176Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:41:56.353Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114139652Z-99b9a8c3--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:41:56.375Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:42:07.912Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114309192Z-3a3cbffd</t>
+  </si>
+  <si>
+    <t>sim-20260913T114309192Z-3a3cbffd--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:43:09.212Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:43:16.205Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114309192Z-3a3cbffd--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:43:16.236Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:43:18.903Z</t>
+  </si>
+  <si>
+    <t>BLOCKED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserContext.newPage: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-SoVWFL --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=879525
+[pid=879525][err] [0913/134317.387100:WARNING:chrome/app/chrome_main_linux.cc:84] Read channel stable from /app/extra/CHROME_VERSION_EXTRA
+[pid=879525] &lt;gracefully close start&gt;</t>
+  </si>
+  <si>
+    <t>sim-20260913T114309192Z-3a3cbffd--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:43:18.914Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:43:28.662Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114415485Z-fd365c0f</t>
+  </si>
+  <si>
+    <t>sim-20260913T114415485Z-fd365c0f--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:44:15.501Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:44:24.896Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114415485Z-fd365c0f--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:44:24.939Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:44:27.366Z</t>
+  </si>
+  <si>
+    <t>browserContext.newPage: Protocol error (Target.createTarget): Failed to open a new tab</t>
+  </si>
+  <si>
+    <t>sim-20260913T114415485Z-fd365c0f--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:44:27.392Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:44:38.630Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114611036Z-4c5127eb</t>
+  </si>
+  <si>
+    <t>sim-20260913T114611036Z-4c5127eb--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:46:11.055Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:46:18.198Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114611036Z-4c5127eb--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:46:18.226Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:46:21.167Z</t>
+  </si>
+  <si>
+    <t>browserContext.newPage: Target page, context or browser has been closed</t>
+  </si>
+  <si>
+    <t>sim-20260913T114611036Z-4c5127eb--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:46:21.202Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:47:21.368Z</t>
+  </si>
+  <si>
+    <t>INTERRUPTED</t>
+  </si>
+  <si>
+    <t>Execució interrompuda detectada durant el resume.</t>
+  </si>
+  <si>
+    <t>sim-20260913T114611036Z-4c5127eb--ZUP-115-DEVELOPER-principal--a02</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:47:21.395Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:47:33.179Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114829506Z-1518f832</t>
+  </si>
+  <si>
+    <t>sim-20260913T114829506Z-1518f832--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:48:29.529Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:48:36.646Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114829506Z-1518f832--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:48:36.697Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:49:26.270Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114829506Z-1518f832--ZUP-073-USER-principal--a02</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:49:26.298Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:49:37.431Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T114829506Z-1518f832--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:49:37.448Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:49:48.001Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T115044005Z-76067d9f</t>
+  </si>
+  <si>
+    <t>sim-20260913T115044005Z-76067d9f--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:50:44.017Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:50:51.577Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T115044005Z-76067d9f--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:50:51.595Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:51:03.431Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T115044005Z-76067d9f--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:51:03.438Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T11:51:13.822Z</t>
   </si>
 </sst>
 </file>
@@ -35431,7 +35836,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -35520,6 +35925,2278 @@
         <v>815</v>
       </c>
     </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>816</v>
+      </c>
+      <c r="B2" t="s">
+        <v>817</v>
+      </c>
+      <c r="C2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" t="s">
+        <v>818</v>
+      </c>
+      <c r="I2" t="s">
+        <v>819</v>
+      </c>
+      <c r="J2" t="s">
+        <v>820</v>
+      </c>
+      <c r="K2" t="s">
+        <v>821</v>
+      </c>
+      <c r="L2" t="s">
+        <v>822</v>
+      </c>
+      <c r="M2" t="s">
+        <v>823</v>
+      </c>
+      <c r="N2">
+        <v>2482</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>825</v>
+      </c>
+      <c r="R2" t="s">
+        <v>825</v>
+      </c>
+      <c r="S2" t="s">
+        <v>826</v>
+      </c>
+      <c r="T2" t="s">
+        <v>825</v>
+      </c>
+      <c r="U2" t="s">
+        <v>827</v>
+      </c>
+      <c r="V2" t="s">
+        <v>820</v>
+      </c>
+      <c r="W2" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>828</v>
+      </c>
+      <c r="B3" t="s">
+        <v>829</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" t="s">
+        <v>818</v>
+      </c>
+      <c r="I3" t="s">
+        <v>819</v>
+      </c>
+      <c r="J3" t="s">
+        <v>820</v>
+      </c>
+      <c r="K3" t="s">
+        <v>821</v>
+      </c>
+      <c r="L3" t="s">
+        <v>830</v>
+      </c>
+      <c r="M3" t="s">
+        <v>831</v>
+      </c>
+      <c r="N3">
+        <v>1621</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>825</v>
+      </c>
+      <c r="R3" t="s">
+        <v>825</v>
+      </c>
+      <c r="S3" t="s">
+        <v>826</v>
+      </c>
+      <c r="T3" t="s">
+        <v>825</v>
+      </c>
+      <c r="U3" t="s">
+        <v>827</v>
+      </c>
+      <c r="V3" t="s">
+        <v>820</v>
+      </c>
+      <c r="W3" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>828</v>
+      </c>
+      <c r="B4" t="s">
+        <v>832</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>427</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" t="s">
+        <v>818</v>
+      </c>
+      <c r="I4" t="s">
+        <v>819</v>
+      </c>
+      <c r="J4" t="s">
+        <v>820</v>
+      </c>
+      <c r="K4" t="s">
+        <v>821</v>
+      </c>
+      <c r="L4" t="s">
+        <v>833</v>
+      </c>
+      <c r="M4" t="s">
+        <v>834</v>
+      </c>
+      <c r="N4">
+        <v>8824</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>825</v>
+      </c>
+      <c r="R4" t="s">
+        <v>825</v>
+      </c>
+      <c r="S4" t="s">
+        <v>836</v>
+      </c>
+      <c r="T4" t="s">
+        <v>837</v>
+      </c>
+      <c r="U4" t="s">
+        <v>827</v>
+      </c>
+      <c r="V4" t="s">
+        <v>820</v>
+      </c>
+      <c r="W4" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>828</v>
+      </c>
+      <c r="B5" t="s">
+        <v>838</v>
+      </c>
+      <c r="C5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" t="s">
+        <v>613</v>
+      </c>
+      <c r="E5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" t="s">
+        <v>818</v>
+      </c>
+      <c r="I5" t="s">
+        <v>819</v>
+      </c>
+      <c r="J5" t="s">
+        <v>820</v>
+      </c>
+      <c r="K5" t="s">
+        <v>821</v>
+      </c>
+      <c r="L5" t="s">
+        <v>839</v>
+      </c>
+      <c r="M5" t="s">
+        <v>840</v>
+      </c>
+      <c r="N5">
+        <v>2540</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>825</v>
+      </c>
+      <c r="R5" t="s">
+        <v>825</v>
+      </c>
+      <c r="S5" t="s">
+        <v>826</v>
+      </c>
+      <c r="T5" t="s">
+        <v>825</v>
+      </c>
+      <c r="U5" t="s">
+        <v>827</v>
+      </c>
+      <c r="V5" t="s">
+        <v>820</v>
+      </c>
+      <c r="W5" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>841</v>
+      </c>
+      <c r="B6" t="s">
+        <v>842</v>
+      </c>
+      <c r="C6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" t="s">
+        <v>427</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H6" t="s">
+        <v>818</v>
+      </c>
+      <c r="I6" t="s">
+        <v>819</v>
+      </c>
+      <c r="J6" t="s">
+        <v>820</v>
+      </c>
+      <c r="K6" t="s">
+        <v>821</v>
+      </c>
+      <c r="L6" t="s">
+        <v>843</v>
+      </c>
+      <c r="M6" t="s">
+        <v>844</v>
+      </c>
+      <c r="N6">
+        <v>2586</v>
+      </c>
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>825</v>
+      </c>
+      <c r="R6" t="s">
+        <v>825</v>
+      </c>
+      <c r="S6" t="s">
+        <v>845</v>
+      </c>
+      <c r="T6" t="s">
+        <v>837</v>
+      </c>
+      <c r="U6" t="s">
+        <v>827</v>
+      </c>
+      <c r="V6" t="s">
+        <v>820</v>
+      </c>
+      <c r="W6" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>846</v>
+      </c>
+      <c r="B7" t="s">
+        <v>847</v>
+      </c>
+      <c r="C7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" t="s">
+        <v>427</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" t="s">
+        <v>818</v>
+      </c>
+      <c r="I7" t="s">
+        <v>819</v>
+      </c>
+      <c r="J7" t="s">
+        <v>820</v>
+      </c>
+      <c r="K7" t="s">
+        <v>821</v>
+      </c>
+      <c r="L7" t="s">
+        <v>848</v>
+      </c>
+      <c r="M7" t="s">
+        <v>849</v>
+      </c>
+      <c r="N7">
+        <v>4373</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>825</v>
+      </c>
+      <c r="R7" t="s">
+        <v>825</v>
+      </c>
+      <c r="S7" t="s">
+        <v>845</v>
+      </c>
+      <c r="T7" t="s">
+        <v>837</v>
+      </c>
+      <c r="U7" t="s">
+        <v>827</v>
+      </c>
+      <c r="V7" t="s">
+        <v>820</v>
+      </c>
+      <c r="W7" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>850</v>
+      </c>
+      <c r="B8" t="s">
+        <v>851</v>
+      </c>
+      <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
+        <v>427</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>64</v>
+      </c>
+      <c r="G8" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" t="s">
+        <v>818</v>
+      </c>
+      <c r="I8" t="s">
+        <v>819</v>
+      </c>
+      <c r="J8" t="s">
+        <v>820</v>
+      </c>
+      <c r="K8" t="s">
+        <v>821</v>
+      </c>
+      <c r="L8" t="s">
+        <v>852</v>
+      </c>
+      <c r="M8" t="s">
+        <v>853</v>
+      </c>
+      <c r="N8">
+        <v>5493</v>
+      </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>825</v>
+      </c>
+      <c r="R8" t="s">
+        <v>825</v>
+      </c>
+      <c r="S8" t="s">
+        <v>845</v>
+      </c>
+      <c r="T8" t="s">
+        <v>837</v>
+      </c>
+      <c r="U8" t="s">
+        <v>827</v>
+      </c>
+      <c r="V8" t="s">
+        <v>820</v>
+      </c>
+      <c r="W8" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>854</v>
+      </c>
+      <c r="B9" t="s">
+        <v>855</v>
+      </c>
+      <c r="C9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" t="s">
+        <v>427</v>
+      </c>
+      <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" t="s">
+        <v>818</v>
+      </c>
+      <c r="I9" t="s">
+        <v>819</v>
+      </c>
+      <c r="J9" t="s">
+        <v>820</v>
+      </c>
+      <c r="K9" t="s">
+        <v>821</v>
+      </c>
+      <c r="L9" t="s">
+        <v>856</v>
+      </c>
+      <c r="M9" t="s">
+        <v>857</v>
+      </c>
+      <c r="N9">
+        <v>7538</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>825</v>
+      </c>
+      <c r="R9" t="s">
+        <v>825</v>
+      </c>
+      <c r="S9" t="s">
+        <v>845</v>
+      </c>
+      <c r="T9" t="s">
+        <v>837</v>
+      </c>
+      <c r="U9" t="s">
+        <v>827</v>
+      </c>
+      <c r="V9" t="s">
+        <v>820</v>
+      </c>
+      <c r="W9" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>858</v>
+      </c>
+      <c r="B10" t="s">
+        <v>859</v>
+      </c>
+      <c r="C10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" t="s">
+        <v>427</v>
+      </c>
+      <c r="E10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H10" t="s">
+        <v>818</v>
+      </c>
+      <c r="I10" t="s">
+        <v>819</v>
+      </c>
+      <c r="J10" t="s">
+        <v>820</v>
+      </c>
+      <c r="K10" t="s">
+        <v>821</v>
+      </c>
+      <c r="L10" t="s">
+        <v>860</v>
+      </c>
+      <c r="M10" t="s">
+        <v>861</v>
+      </c>
+      <c r="N10">
+        <v>13972</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>825</v>
+      </c>
+      <c r="R10" t="s">
+        <v>825</v>
+      </c>
+      <c r="S10" t="s">
+        <v>826</v>
+      </c>
+      <c r="T10" t="s">
+        <v>825</v>
+      </c>
+      <c r="U10" t="s">
+        <v>827</v>
+      </c>
+      <c r="V10" t="s">
+        <v>820</v>
+      </c>
+      <c r="W10" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>862</v>
+      </c>
+      <c r="B11" t="s">
+        <v>863</v>
+      </c>
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" t="s">
+        <v>427</v>
+      </c>
+      <c r="E11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" t="s">
+        <v>818</v>
+      </c>
+      <c r="I11" t="s">
+        <v>819</v>
+      </c>
+      <c r="J11" t="s">
+        <v>820</v>
+      </c>
+      <c r="K11" t="s">
+        <v>821</v>
+      </c>
+      <c r="L11" t="s">
+        <v>864</v>
+      </c>
+      <c r="M11" t="s">
+        <v>865</v>
+      </c>
+      <c r="N11">
+        <v>13228</v>
+      </c>
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>825</v>
+      </c>
+      <c r="R11" t="s">
+        <v>825</v>
+      </c>
+      <c r="S11" t="s">
+        <v>826</v>
+      </c>
+      <c r="T11" t="s">
+        <v>825</v>
+      </c>
+      <c r="U11" t="s">
+        <v>827</v>
+      </c>
+      <c r="V11" t="s">
+        <v>820</v>
+      </c>
+      <c r="W11" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>866</v>
+      </c>
+      <c r="B12" t="s">
+        <v>867</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>427</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" t="s">
+        <v>818</v>
+      </c>
+      <c r="I12" t="s">
+        <v>819</v>
+      </c>
+      <c r="J12" t="s">
+        <v>820</v>
+      </c>
+      <c r="K12" t="s">
+        <v>821</v>
+      </c>
+      <c r="L12" t="s">
+        <v>868</v>
+      </c>
+      <c r="M12" t="s">
+        <v>869</v>
+      </c>
+      <c r="N12">
+        <v>11819</v>
+      </c>
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>825</v>
+      </c>
+      <c r="R12" t="s">
+        <v>825</v>
+      </c>
+      <c r="S12" t="s">
+        <v>826</v>
+      </c>
+      <c r="T12" t="s">
+        <v>825</v>
+      </c>
+      <c r="U12" t="s">
+        <v>827</v>
+      </c>
+      <c r="V12" t="s">
+        <v>820</v>
+      </c>
+      <c r="W12" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>870</v>
+      </c>
+      <c r="B13" t="s">
+        <v>871</v>
+      </c>
+      <c r="C13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" t="s">
+        <v>427</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" t="s">
+        <v>64</v>
+      </c>
+      <c r="G13" t="s">
+        <v>60</v>
+      </c>
+      <c r="H13" t="s">
+        <v>818</v>
+      </c>
+      <c r="I13" t="s">
+        <v>819</v>
+      </c>
+      <c r="J13" t="s">
+        <v>820</v>
+      </c>
+      <c r="K13" t="s">
+        <v>821</v>
+      </c>
+      <c r="L13" t="s">
+        <v>872</v>
+      </c>
+      <c r="M13" t="s">
+        <v>873</v>
+      </c>
+      <c r="N13">
+        <v>12833</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>825</v>
+      </c>
+      <c r="R13" t="s">
+        <v>825</v>
+      </c>
+      <c r="S13" t="s">
+        <v>826</v>
+      </c>
+      <c r="T13" t="s">
+        <v>825</v>
+      </c>
+      <c r="U13" t="s">
+        <v>827</v>
+      </c>
+      <c r="V13" t="s">
+        <v>820</v>
+      </c>
+      <c r="W13" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>874</v>
+      </c>
+      <c r="B14" t="s">
+        <v>875</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>61</v>
+      </c>
+      <c r="F14" t="s">
+        <v>64</v>
+      </c>
+      <c r="G14" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" t="s">
+        <v>818</v>
+      </c>
+      <c r="I14" t="s">
+        <v>819</v>
+      </c>
+      <c r="J14" t="s">
+        <v>820</v>
+      </c>
+      <c r="K14" t="s">
+        <v>821</v>
+      </c>
+      <c r="L14" t="s">
+        <v>876</v>
+      </c>
+      <c r="M14" t="s">
+        <v>877</v>
+      </c>
+      <c r="N14">
+        <v>6398</v>
+      </c>
+      <c r="O14">
+        <v>1</v>
+      </c>
+      <c r="P14" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>825</v>
+      </c>
+      <c r="R14" t="s">
+        <v>825</v>
+      </c>
+      <c r="S14" t="s">
+        <v>826</v>
+      </c>
+      <c r="T14" t="s">
+        <v>825</v>
+      </c>
+      <c r="U14" t="s">
+        <v>827</v>
+      </c>
+      <c r="V14" t="s">
+        <v>820</v>
+      </c>
+      <c r="W14" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>874</v>
+      </c>
+      <c r="B15" t="s">
+        <v>878</v>
+      </c>
+      <c r="C15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" t="s">
+        <v>427</v>
+      </c>
+      <c r="E15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H15" t="s">
+        <v>818</v>
+      </c>
+      <c r="I15" t="s">
+        <v>819</v>
+      </c>
+      <c r="J15" t="s">
+        <v>820</v>
+      </c>
+      <c r="K15" t="s">
+        <v>821</v>
+      </c>
+      <c r="L15" t="s">
+        <v>879</v>
+      </c>
+      <c r="M15" t="s">
+        <v>880</v>
+      </c>
+      <c r="N15">
+        <v>10177</v>
+      </c>
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>825</v>
+      </c>
+      <c r="R15" t="s">
+        <v>825</v>
+      </c>
+      <c r="S15" t="s">
+        <v>826</v>
+      </c>
+      <c r="T15" t="s">
+        <v>825</v>
+      </c>
+      <c r="U15" t="s">
+        <v>827</v>
+      </c>
+      <c r="V15" t="s">
+        <v>820</v>
+      </c>
+      <c r="W15" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>874</v>
+      </c>
+      <c r="B16" t="s">
+        <v>881</v>
+      </c>
+      <c r="C16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" t="s">
+        <v>613</v>
+      </c>
+      <c r="E16" t="s">
+        <v>188</v>
+      </c>
+      <c r="F16" t="s">
+        <v>64</v>
+      </c>
+      <c r="G16" t="s">
+        <v>60</v>
+      </c>
+      <c r="H16" t="s">
+        <v>818</v>
+      </c>
+      <c r="I16" t="s">
+        <v>819</v>
+      </c>
+      <c r="J16" t="s">
+        <v>820</v>
+      </c>
+      <c r="K16" t="s">
+        <v>821</v>
+      </c>
+      <c r="L16" t="s">
+        <v>882</v>
+      </c>
+      <c r="M16" t="s">
+        <v>883</v>
+      </c>
+      <c r="N16">
+        <v>11537</v>
+      </c>
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>825</v>
+      </c>
+      <c r="R16" t="s">
+        <v>825</v>
+      </c>
+      <c r="S16" t="s">
+        <v>826</v>
+      </c>
+      <c r="T16" t="s">
+        <v>825</v>
+      </c>
+      <c r="U16" t="s">
+        <v>827</v>
+      </c>
+      <c r="V16" t="s">
+        <v>820</v>
+      </c>
+      <c r="W16" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>884</v>
+      </c>
+      <c r="B17" t="s">
+        <v>885</v>
+      </c>
+      <c r="C17" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" t="s">
+        <v>60</v>
+      </c>
+      <c r="H17" t="s">
+        <v>818</v>
+      </c>
+      <c r="I17" t="s">
+        <v>819</v>
+      </c>
+      <c r="J17" t="s">
+        <v>820</v>
+      </c>
+      <c r="K17" t="s">
+        <v>821</v>
+      </c>
+      <c r="L17" t="s">
+        <v>886</v>
+      </c>
+      <c r="M17" t="s">
+        <v>887</v>
+      </c>
+      <c r="N17">
+        <v>6993</v>
+      </c>
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>825</v>
+      </c>
+      <c r="R17" t="s">
+        <v>825</v>
+      </c>
+      <c r="S17" t="s">
+        <v>826</v>
+      </c>
+      <c r="T17" t="s">
+        <v>825</v>
+      </c>
+      <c r="U17" t="s">
+        <v>827</v>
+      </c>
+      <c r="V17" t="s">
+        <v>820</v>
+      </c>
+      <c r="W17" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>884</v>
+      </c>
+      <c r="B18" t="s">
+        <v>888</v>
+      </c>
+      <c r="C18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" t="s">
+        <v>427</v>
+      </c>
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H18" t="s">
+        <v>818</v>
+      </c>
+      <c r="I18" t="s">
+        <v>819</v>
+      </c>
+      <c r="J18" t="s">
+        <v>820</v>
+      </c>
+      <c r="K18" t="s">
+        <v>821</v>
+      </c>
+      <c r="L18" t="s">
+        <v>889</v>
+      </c>
+      <c r="M18" t="s">
+        <v>890</v>
+      </c>
+      <c r="N18">
+        <v>2667</v>
+      </c>
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>825</v>
+      </c>
+      <c r="R18" t="s">
+        <v>825</v>
+      </c>
+      <c r="S18" t="s">
+        <v>892</v>
+      </c>
+      <c r="T18" t="s">
+        <v>837</v>
+      </c>
+      <c r="U18" t="s">
+        <v>827</v>
+      </c>
+      <c r="V18" t="s">
+        <v>820</v>
+      </c>
+      <c r="W18" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>884</v>
+      </c>
+      <c r="B19" t="s">
+        <v>893</v>
+      </c>
+      <c r="C19" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" t="s">
+        <v>613</v>
+      </c>
+      <c r="E19" t="s">
+        <v>188</v>
+      </c>
+      <c r="F19" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" t="s">
+        <v>60</v>
+      </c>
+      <c r="H19" t="s">
+        <v>818</v>
+      </c>
+      <c r="I19" t="s">
+        <v>819</v>
+      </c>
+      <c r="J19" t="s">
+        <v>820</v>
+      </c>
+      <c r="K19" t="s">
+        <v>821</v>
+      </c>
+      <c r="L19" t="s">
+        <v>894</v>
+      </c>
+      <c r="M19" t="s">
+        <v>895</v>
+      </c>
+      <c r="N19">
+        <v>9748</v>
+      </c>
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>825</v>
+      </c>
+      <c r="R19" t="s">
+        <v>825</v>
+      </c>
+      <c r="S19" t="s">
+        <v>826</v>
+      </c>
+      <c r="T19" t="s">
+        <v>825</v>
+      </c>
+      <c r="U19" t="s">
+        <v>827</v>
+      </c>
+      <c r="V19" t="s">
+        <v>820</v>
+      </c>
+      <c r="W19" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>896</v>
+      </c>
+      <c r="B20" t="s">
+        <v>897</v>
+      </c>
+      <c r="C20" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20" t="s">
+        <v>60</v>
+      </c>
+      <c r="H20" t="s">
+        <v>818</v>
+      </c>
+      <c r="I20" t="s">
+        <v>819</v>
+      </c>
+      <c r="J20" t="s">
+        <v>820</v>
+      </c>
+      <c r="K20" t="s">
+        <v>821</v>
+      </c>
+      <c r="L20" t="s">
+        <v>898</v>
+      </c>
+      <c r="M20" t="s">
+        <v>899</v>
+      </c>
+      <c r="N20">
+        <v>9395</v>
+      </c>
+      <c r="O20">
+        <v>1</v>
+      </c>
+      <c r="P20" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>825</v>
+      </c>
+      <c r="R20" t="s">
+        <v>825</v>
+      </c>
+      <c r="S20" t="s">
+        <v>826</v>
+      </c>
+      <c r="T20" t="s">
+        <v>825</v>
+      </c>
+      <c r="U20" t="s">
+        <v>827</v>
+      </c>
+      <c r="V20" t="s">
+        <v>820</v>
+      </c>
+      <c r="W20" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>896</v>
+      </c>
+      <c r="B21" t="s">
+        <v>900</v>
+      </c>
+      <c r="C21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" t="s">
+        <v>427</v>
+      </c>
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" t="s">
+        <v>60</v>
+      </c>
+      <c r="H21" t="s">
+        <v>818</v>
+      </c>
+      <c r="I21" t="s">
+        <v>819</v>
+      </c>
+      <c r="J21" t="s">
+        <v>820</v>
+      </c>
+      <c r="K21" t="s">
+        <v>821</v>
+      </c>
+      <c r="L21" t="s">
+        <v>901</v>
+      </c>
+      <c r="M21" t="s">
+        <v>902</v>
+      </c>
+      <c r="N21">
+        <v>2427</v>
+      </c>
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>825</v>
+      </c>
+      <c r="R21" t="s">
+        <v>825</v>
+      </c>
+      <c r="S21" t="s">
+        <v>903</v>
+      </c>
+      <c r="T21" t="s">
+        <v>837</v>
+      </c>
+      <c r="U21" t="s">
+        <v>827</v>
+      </c>
+      <c r="V21" t="s">
+        <v>820</v>
+      </c>
+      <c r="W21" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>896</v>
+      </c>
+      <c r="B22" t="s">
+        <v>904</v>
+      </c>
+      <c r="C22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" t="s">
+        <v>613</v>
+      </c>
+      <c r="E22" t="s">
+        <v>188</v>
+      </c>
+      <c r="F22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" t="s">
+        <v>60</v>
+      </c>
+      <c r="H22" t="s">
+        <v>818</v>
+      </c>
+      <c r="I22" t="s">
+        <v>819</v>
+      </c>
+      <c r="J22" t="s">
+        <v>820</v>
+      </c>
+      <c r="K22" t="s">
+        <v>821</v>
+      </c>
+      <c r="L22" t="s">
+        <v>905</v>
+      </c>
+      <c r="M22" t="s">
+        <v>906</v>
+      </c>
+      <c r="N22">
+        <v>11238</v>
+      </c>
+      <c r="O22">
+        <v>1</v>
+      </c>
+      <c r="P22" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>825</v>
+      </c>
+      <c r="R22" t="s">
+        <v>825</v>
+      </c>
+      <c r="S22" t="s">
+        <v>826</v>
+      </c>
+      <c r="T22" t="s">
+        <v>825</v>
+      </c>
+      <c r="U22" t="s">
+        <v>827</v>
+      </c>
+      <c r="V22" t="s">
+        <v>820</v>
+      </c>
+      <c r="W22" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>907</v>
+      </c>
+      <c r="B23" t="s">
+        <v>908</v>
+      </c>
+      <c r="C23" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" t="s">
+        <v>61</v>
+      </c>
+      <c r="F23" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" t="s">
+        <v>60</v>
+      </c>
+      <c r="H23" t="s">
+        <v>818</v>
+      </c>
+      <c r="I23" t="s">
+        <v>819</v>
+      </c>
+      <c r="J23" t="s">
+        <v>820</v>
+      </c>
+      <c r="K23" t="s">
+        <v>821</v>
+      </c>
+      <c r="L23" t="s">
+        <v>909</v>
+      </c>
+      <c r="M23" t="s">
+        <v>910</v>
+      </c>
+      <c r="N23">
+        <v>7143</v>
+      </c>
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>825</v>
+      </c>
+      <c r="R23" t="s">
+        <v>825</v>
+      </c>
+      <c r="S23" t="s">
+        <v>826</v>
+      </c>
+      <c r="T23" t="s">
+        <v>825</v>
+      </c>
+      <c r="U23" t="s">
+        <v>827</v>
+      </c>
+      <c r="V23" t="s">
+        <v>820</v>
+      </c>
+      <c r="W23" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>907</v>
+      </c>
+      <c r="B24" t="s">
+        <v>911</v>
+      </c>
+      <c r="C24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" t="s">
+        <v>427</v>
+      </c>
+      <c r="E24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" t="s">
+        <v>60</v>
+      </c>
+      <c r="H24" t="s">
+        <v>818</v>
+      </c>
+      <c r="I24" t="s">
+        <v>819</v>
+      </c>
+      <c r="J24" t="s">
+        <v>820</v>
+      </c>
+      <c r="K24" t="s">
+        <v>821</v>
+      </c>
+      <c r="L24" t="s">
+        <v>912</v>
+      </c>
+      <c r="M24" t="s">
+        <v>913</v>
+      </c>
+      <c r="N24">
+        <v>2941</v>
+      </c>
+      <c r="O24">
+        <v>1</v>
+      </c>
+      <c r="P24" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>825</v>
+      </c>
+      <c r="R24" t="s">
+        <v>825</v>
+      </c>
+      <c r="S24" t="s">
+        <v>914</v>
+      </c>
+      <c r="T24" t="s">
+        <v>825</v>
+      </c>
+      <c r="U24" t="s">
+        <v>827</v>
+      </c>
+      <c r="V24" t="s">
+        <v>820</v>
+      </c>
+      <c r="W24" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>907</v>
+      </c>
+      <c r="B25" t="s">
+        <v>915</v>
+      </c>
+      <c r="C25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" t="s">
+        <v>613</v>
+      </c>
+      <c r="E25" t="s">
+        <v>188</v>
+      </c>
+      <c r="F25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G25" t="s">
+        <v>60</v>
+      </c>
+      <c r="H25" t="s">
+        <v>818</v>
+      </c>
+      <c r="I25" t="s">
+        <v>819</v>
+      </c>
+      <c r="J25" t="s">
+        <v>820</v>
+      </c>
+      <c r="K25" t="s">
+        <v>821</v>
+      </c>
+      <c r="L25" t="s">
+        <v>916</v>
+      </c>
+      <c r="M25" t="s">
+        <v>917</v>
+      </c>
+      <c r="N25">
+        <v>60166</v>
+      </c>
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25" t="s">
+        <v>918</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>825</v>
+      </c>
+      <c r="R25" t="s">
+        <v>825</v>
+      </c>
+      <c r="S25" t="s">
+        <v>919</v>
+      </c>
+      <c r="T25" t="s">
+        <v>825</v>
+      </c>
+      <c r="U25" t="s">
+        <v>827</v>
+      </c>
+      <c r="V25" t="s">
+        <v>820</v>
+      </c>
+      <c r="W25" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>907</v>
+      </c>
+      <c r="B26" t="s">
+        <v>920</v>
+      </c>
+      <c r="C26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" t="s">
+        <v>613</v>
+      </c>
+      <c r="E26" t="s">
+        <v>188</v>
+      </c>
+      <c r="F26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" t="s">
+        <v>60</v>
+      </c>
+      <c r="H26" t="s">
+        <v>818</v>
+      </c>
+      <c r="I26" t="s">
+        <v>819</v>
+      </c>
+      <c r="J26" t="s">
+        <v>820</v>
+      </c>
+      <c r="K26" t="s">
+        <v>821</v>
+      </c>
+      <c r="L26" t="s">
+        <v>921</v>
+      </c>
+      <c r="M26" t="s">
+        <v>922</v>
+      </c>
+      <c r="N26">
+        <v>11784</v>
+      </c>
+      <c r="O26">
+        <v>2</v>
+      </c>
+      <c r="P26" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>825</v>
+      </c>
+      <c r="R26" t="s">
+        <v>825</v>
+      </c>
+      <c r="S26" t="s">
+        <v>826</v>
+      </c>
+      <c r="T26" t="s">
+        <v>825</v>
+      </c>
+      <c r="U26" t="s">
+        <v>827</v>
+      </c>
+      <c r="V26" t="s">
+        <v>820</v>
+      </c>
+      <c r="W26" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>923</v>
+      </c>
+      <c r="B27" t="s">
+        <v>924</v>
+      </c>
+      <c r="C27" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" t="s">
+        <v>64</v>
+      </c>
+      <c r="G27" t="s">
+        <v>60</v>
+      </c>
+      <c r="H27" t="s">
+        <v>818</v>
+      </c>
+      <c r="I27" t="s">
+        <v>819</v>
+      </c>
+      <c r="J27" t="s">
+        <v>820</v>
+      </c>
+      <c r="K27" t="s">
+        <v>821</v>
+      </c>
+      <c r="L27" t="s">
+        <v>925</v>
+      </c>
+      <c r="M27" t="s">
+        <v>926</v>
+      </c>
+      <c r="N27">
+        <v>7117</v>
+      </c>
+      <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>825</v>
+      </c>
+      <c r="R27" t="s">
+        <v>825</v>
+      </c>
+      <c r="S27" t="s">
+        <v>826</v>
+      </c>
+      <c r="T27" t="s">
+        <v>825</v>
+      </c>
+      <c r="U27" t="s">
+        <v>827</v>
+      </c>
+      <c r="V27" t="s">
+        <v>820</v>
+      </c>
+      <c r="W27" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>923</v>
+      </c>
+      <c r="B28" t="s">
+        <v>927</v>
+      </c>
+      <c r="C28" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" t="s">
+        <v>427</v>
+      </c>
+      <c r="E28" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28" t="s">
+        <v>64</v>
+      </c>
+      <c r="G28" t="s">
+        <v>60</v>
+      </c>
+      <c r="H28" t="s">
+        <v>818</v>
+      </c>
+      <c r="I28" t="s">
+        <v>819</v>
+      </c>
+      <c r="J28" t="s">
+        <v>820</v>
+      </c>
+      <c r="K28" t="s">
+        <v>821</v>
+      </c>
+      <c r="L28" t="s">
+        <v>928</v>
+      </c>
+      <c r="M28" t="s">
+        <v>929</v>
+      </c>
+      <c r="N28">
+        <v>49573</v>
+      </c>
+      <c r="O28">
+        <v>1</v>
+      </c>
+      <c r="P28" t="s">
+        <v>918</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>825</v>
+      </c>
+      <c r="R28" t="s">
+        <v>825</v>
+      </c>
+      <c r="S28" t="s">
+        <v>919</v>
+      </c>
+      <c r="T28" t="s">
+        <v>825</v>
+      </c>
+      <c r="U28" t="s">
+        <v>827</v>
+      </c>
+      <c r="V28" t="s">
+        <v>820</v>
+      </c>
+      <c r="W28" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>923</v>
+      </c>
+      <c r="B29" t="s">
+        <v>930</v>
+      </c>
+      <c r="C29" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" t="s">
+        <v>427</v>
+      </c>
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+      <c r="F29" t="s">
+        <v>64</v>
+      </c>
+      <c r="G29" t="s">
+        <v>60</v>
+      </c>
+      <c r="H29" t="s">
+        <v>818</v>
+      </c>
+      <c r="I29" t="s">
+        <v>819</v>
+      </c>
+      <c r="J29" t="s">
+        <v>820</v>
+      </c>
+      <c r="K29" t="s">
+        <v>821</v>
+      </c>
+      <c r="L29" t="s">
+        <v>931</v>
+      </c>
+      <c r="M29" t="s">
+        <v>932</v>
+      </c>
+      <c r="N29">
+        <v>11133</v>
+      </c>
+      <c r="O29">
+        <v>2</v>
+      </c>
+      <c r="P29" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>825</v>
+      </c>
+      <c r="R29" t="s">
+        <v>825</v>
+      </c>
+      <c r="S29" t="s">
+        <v>826</v>
+      </c>
+      <c r="T29" t="s">
+        <v>825</v>
+      </c>
+      <c r="U29" t="s">
+        <v>827</v>
+      </c>
+      <c r="V29" t="s">
+        <v>820</v>
+      </c>
+      <c r="W29" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>923</v>
+      </c>
+      <c r="B30" t="s">
+        <v>933</v>
+      </c>
+      <c r="C30" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" t="s">
+        <v>613</v>
+      </c>
+      <c r="E30" t="s">
+        <v>188</v>
+      </c>
+      <c r="F30" t="s">
+        <v>64</v>
+      </c>
+      <c r="G30" t="s">
+        <v>60</v>
+      </c>
+      <c r="H30" t="s">
+        <v>818</v>
+      </c>
+      <c r="I30" t="s">
+        <v>819</v>
+      </c>
+      <c r="J30" t="s">
+        <v>820</v>
+      </c>
+      <c r="K30" t="s">
+        <v>821</v>
+      </c>
+      <c r="L30" t="s">
+        <v>934</v>
+      </c>
+      <c r="M30" t="s">
+        <v>935</v>
+      </c>
+      <c r="N30">
+        <v>10553</v>
+      </c>
+      <c r="O30">
+        <v>1</v>
+      </c>
+      <c r="P30" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>825</v>
+      </c>
+      <c r="R30" t="s">
+        <v>825</v>
+      </c>
+      <c r="S30" t="s">
+        <v>826</v>
+      </c>
+      <c r="T30" t="s">
+        <v>825</v>
+      </c>
+      <c r="U30" t="s">
+        <v>827</v>
+      </c>
+      <c r="V30" t="s">
+        <v>820</v>
+      </c>
+      <c r="W30" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>936</v>
+      </c>
+      <c r="B31" t="s">
+        <v>937</v>
+      </c>
+      <c r="C31" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" t="s">
+        <v>56</v>
+      </c>
+      <c r="E31" t="s">
+        <v>61</v>
+      </c>
+      <c r="F31" t="s">
+        <v>64</v>
+      </c>
+      <c r="G31" t="s">
+        <v>60</v>
+      </c>
+      <c r="H31" t="s">
+        <v>818</v>
+      </c>
+      <c r="I31" t="s">
+        <v>819</v>
+      </c>
+      <c r="J31" t="s">
+        <v>820</v>
+      </c>
+      <c r="K31" t="s">
+        <v>821</v>
+      </c>
+      <c r="L31" t="s">
+        <v>938</v>
+      </c>
+      <c r="M31" t="s">
+        <v>939</v>
+      </c>
+      <c r="N31">
+        <v>7560</v>
+      </c>
+      <c r="O31">
+        <v>1</v>
+      </c>
+      <c r="P31" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>825</v>
+      </c>
+      <c r="R31" t="s">
+        <v>825</v>
+      </c>
+      <c r="S31" t="s">
+        <v>826</v>
+      </c>
+      <c r="T31" t="s">
+        <v>825</v>
+      </c>
+      <c r="U31" t="s">
+        <v>827</v>
+      </c>
+      <c r="V31" t="s">
+        <v>820</v>
+      </c>
+      <c r="W31" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>936</v>
+      </c>
+      <c r="B32" t="s">
+        <v>940</v>
+      </c>
+      <c r="C32" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" t="s">
+        <v>427</v>
+      </c>
+      <c r="E32" t="s">
+        <v>34</v>
+      </c>
+      <c r="F32" t="s">
+        <v>64</v>
+      </c>
+      <c r="G32" t="s">
+        <v>60</v>
+      </c>
+      <c r="H32" t="s">
+        <v>818</v>
+      </c>
+      <c r="I32" t="s">
+        <v>819</v>
+      </c>
+      <c r="J32" t="s">
+        <v>820</v>
+      </c>
+      <c r="K32" t="s">
+        <v>821</v>
+      </c>
+      <c r="L32" t="s">
+        <v>941</v>
+      </c>
+      <c r="M32" t="s">
+        <v>942</v>
+      </c>
+      <c r="N32">
+        <v>11836</v>
+      </c>
+      <c r="O32">
+        <v>1</v>
+      </c>
+      <c r="P32" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>825</v>
+      </c>
+      <c r="R32" t="s">
+        <v>825</v>
+      </c>
+      <c r="S32" t="s">
+        <v>826</v>
+      </c>
+      <c r="T32" t="s">
+        <v>825</v>
+      </c>
+      <c r="U32" t="s">
+        <v>827</v>
+      </c>
+      <c r="V32" t="s">
+        <v>820</v>
+      </c>
+      <c r="W32" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>936</v>
+      </c>
+      <c r="B33" t="s">
+        <v>943</v>
+      </c>
+      <c r="C33" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" t="s">
+        <v>613</v>
+      </c>
+      <c r="E33" t="s">
+        <v>188</v>
+      </c>
+      <c r="F33" t="s">
+        <v>64</v>
+      </c>
+      <c r="G33" t="s">
+        <v>60</v>
+      </c>
+      <c r="H33" t="s">
+        <v>818</v>
+      </c>
+      <c r="I33" t="s">
+        <v>819</v>
+      </c>
+      <c r="J33" t="s">
+        <v>820</v>
+      </c>
+      <c r="K33" t="s">
+        <v>821</v>
+      </c>
+      <c r="L33" t="s">
+        <v>944</v>
+      </c>
+      <c r="M33" t="s">
+        <v>945</v>
+      </c>
+      <c r="N33">
+        <v>10384</v>
+      </c>
+      <c r="O33">
+        <v>1</v>
+      </c>
+      <c r="P33" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>825</v>
+      </c>
+      <c r="R33" t="s">
+        <v>825</v>
+      </c>
+      <c r="S33" t="s">
+        <v>826</v>
+      </c>
+      <c r="T33" t="s">
+        <v>825</v>
+      </c>
+      <c r="U33" t="s">
+        <v>827</v>
+      </c>
+      <c r="V33" t="s">
+        <v>820</v>
+      </c>
+      <c r="W33" t="s">
+        <v>825</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
116 ⇒ fase IV ⇒ E2E Fase IV: fixtures, factories, cleanup i rols validats
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6491" uniqueCount="946">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7373" uniqueCount="1113">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -2995,6 +2995,805 @@
   </si>
   <si>
     <t>2026-09-13T11:51:13.822Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T200448216Z-7bfb8ff2</t>
+  </si>
+  <si>
+    <t>sim-20260913T200448216Z-7bfb8ff2--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>unknown</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:04:48.226Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:04:48.322Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-gyygtm --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=62
+[pid=62][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-gyygtm --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=62[22m
+[2m  - [pid=62][err] error: Unable to allocate instance id[22m
+[2m  - [pid=62] &lt;gracefully close start&gt;[22m
+[2m  - [pid=62] &lt;kill&gt;[22m
+[2m  - [pid=62] &lt;will force kill&gt;[22m
+[2m  - [pid=62] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=62] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=62] starting temporary directories cleanup[22m
+[2m  - [pid=62] finished temporary directories cleanup[22m
+[2m  - [pid=62] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>/DATA/repos/zuppeto/e2e/.runs/artifacts/ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>sim-20260913T200448216Z-7bfb8ff2--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:04:48.330Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:04:48.380Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-0WPEsb --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=65
+[pid=65][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-0WPEsb --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=65[22m
+[2m  - [pid=65][err] error: Unable to allocate instance id[22m
+[2m  - [pid=65] &lt;gracefully close start&gt;[22m
+[2m  - [pid=65] &lt;kill&gt;[22m
+[2m  - [pid=65] &lt;will force kill&gt;[22m
+[2m  - [pid=65] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=65] starting temporary directories cleanup[22m
+[2m  - [pid=65] finished temporary directories cleanup[22m
+[2m  - [pid=65] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T200448216Z-7bfb8ff2--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:04:48.385Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:04:48.437Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-heijAG --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=68
+[pid=68][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-heijAG --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=68[22m
+[2m  - [pid=68][err] error: Unable to allocate instance id[22m
+[2m  - [pid=68] &lt;gracefully close start&gt;[22m
+[2m  - [pid=68] &lt;kill&gt;[22m
+[2m  - [pid=68] &lt;will force kill&gt;[22m
+[2m  - [pid=68] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=68] starting temporary directories cleanup[22m
+[2m  - [pid=68] finished temporary directories cleanup[22m
+[2m  - [pid=68] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>/DATA/repos/zuppeto/e2e/.runs/artifacts/ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>sim-20260913T201123046Z-3494803f</t>
+  </si>
+  <si>
+    <t>sim-20260913T201123046Z-3494803f--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:23.052Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:23.131Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-Dkfum0 --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=62
+[pid=62][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-Dkfum0 --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=62[22m
+[2m  - [pid=62][err] error: Unable to allocate instance id[22m
+[2m  - [pid=62] &lt;gracefully close start&gt;[22m
+[2m  - [pid=62] &lt;kill&gt;[22m
+[2m  - [pid=62] &lt;will force kill&gt;[22m
+[2m  - [pid=62] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=62] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=62] starting temporary directories cleanup[22m
+[2m  - [pid=62] finished temporary directories cleanup[22m
+[2m  - [pid=62] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201123046Z-3494803f--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:23.136Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:23.193Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-72H4Av --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=65
+[pid=65][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-72H4Av --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=65[22m
+[2m  - [pid=65][err] error: Unable to allocate instance id[22m
+[2m  - [pid=65] &lt;gracefully close start&gt;[22m
+[2m  - [pid=65] &lt;kill&gt;[22m
+[2m  - [pid=65] &lt;will force kill&gt;[22m
+[2m  - [pid=65] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=65] starting temporary directories cleanup[22m
+[2m  - [pid=65] finished temporary directories cleanup[22m
+[2m  - [pid=65] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201123046Z-3494803f--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:23.201Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:23.256Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-pfamBT --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=68
+[pid=68][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-pfamBT --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=68[22m
+[2m  - [pid=68][err] error: Unable to allocate instance id[22m
+[2m  - [pid=68] &lt;gracefully close start&gt;[22m
+[2m  - [pid=68] &lt;kill&gt;[22m
+[2m  - [pid=68] &lt;will force kill&gt;[22m
+[2m  - [pid=68] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=68] starting temporary directories cleanup[22m
+[2m  - [pid=68] finished temporary directories cleanup[22m
+[2m  - [pid=68] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201141086Z-4cbd030a</t>
+  </si>
+  <si>
+    <t>sim-20260913T201141086Z-4cbd030a--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:41.090Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:41.147Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-GEjvbI --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=63
+[pid=63][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-GEjvbI --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=63[22m
+[2m  - [pid=63][err] error: Unable to allocate instance id[22m
+[2m  - [pid=63] &lt;gracefully close start&gt;[22m
+[2m  - [pid=63] &lt;kill&gt;[22m
+[2m  - [pid=63] &lt;will force kill&gt;[22m
+[2m  - [pid=63] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=63] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=63] starting temporary directories cleanup[22m
+[2m  - [pid=63] finished temporary directories cleanup[22m
+[2m  - [pid=63] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201141086Z-4cbd030a--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:41.151Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:41.186Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-dtbJ7x --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=66
+[pid=66][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-dtbJ7x --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=66[22m
+[2m  - [pid=66][err] error: Unable to allocate instance id[22m
+[2m  - [pid=66] &lt;gracefully close start&gt;[22m
+[2m  - [pid=66] &lt;kill&gt;[22m
+[2m  - [pid=66] &lt;will force kill&gt;[22m
+[2m  - [pid=66] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=66] starting temporary directories cleanup[22m
+[2m  - [pid=66] finished temporary directories cleanup[22m
+[2m  - [pid=66] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201141086Z-4cbd030a--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:41.190Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:41.225Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-YLW0QN --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=69
+[pid=69][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-YLW0QN --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=69[22m
+[2m  - [pid=69][err] error: Unable to allocate instance id[22m
+[2m  - [pid=69] &lt;gracefully close start&gt;[22m
+[2m  - [pid=69] &lt;kill&gt;[22m
+[2m  - [pid=69] &lt;will force kill&gt;[22m
+[2m  - [pid=69] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=69] starting temporary directories cleanup[22m
+[2m  - [pid=69] finished temporary directories cleanup[22m
+[2m  - [pid=69] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201148603Z-21aa6dd1</t>
+  </si>
+  <si>
+    <t>sim-20260913T201148603Z-21aa6dd1--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:48.608Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:48.703Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-q6CW6e --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=113
+[pid=113][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-q6CW6e --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=113[22m
+[2m  - [pid=113][err] error: Unable to allocate instance id[22m
+[2m  - [pid=113] &lt;gracefully close start&gt;[22m
+[2m  - [pid=113] &lt;kill&gt;[22m
+[2m  - [pid=113] &lt;will force kill&gt;[22m
+[2m  - [pid=113] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=113] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=113] starting temporary directories cleanup[22m
+[2m  - [pid=113] finished temporary directories cleanup[22m
+[2m  - [pid=113] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201148603Z-21aa6dd1--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:48.708Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:48.750Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-humG61 --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=116
+[pid=116][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-humG61 --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=116[22m
+[2m  - [pid=116][err] error: Unable to allocate instance id[22m
+[2m  - [pid=116] &lt;gracefully close start&gt;[22m
+[2m  - [pid=116] &lt;kill&gt;[22m
+[2m  - [pid=116] &lt;will force kill&gt;[22m
+[2m  - [pid=116] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=116] starting temporary directories cleanup[22m
+[2m  - [pid=116] finished temporary directories cleanup[22m
+[2m  - [pid=116] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201148603Z-21aa6dd1--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:48.754Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:48.793Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-rLxKtS --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=119
+[pid=119][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-rLxKtS --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=119[22m
+[2m  - [pid=119][err] error: Unable to allocate instance id[22m
+[2m  - [pid=119] &lt;gracefully close start&gt;[22m
+[2m  - [pid=119] &lt;kill&gt;[22m
+[2m  - [pid=119] &lt;will force kill&gt;[22m
+[2m  - [pid=119] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=119] starting temporary directories cleanup[22m
+[2m  - [pid=119] finished temporary directories cleanup[22m
+[2m  - [pid=119] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201157633Z-830580a6</t>
+  </si>
+  <si>
+    <t>sim-20260913T201157633Z-830580a6--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:57.638Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:57.695Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-DOMt1c --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=162
+[pid=162][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-DOMt1c --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=162[22m
+[2m  - [pid=162][err] error: Unable to allocate instance id[22m
+[2m  - [pid=162] &lt;gracefully close start&gt;[22m
+[2m  - [pid=162] &lt;kill&gt;[22m
+[2m  - [pid=162] &lt;will force kill&gt;[22m
+[2m  - [pid=162] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=162] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=162] starting temporary directories cleanup[22m
+[2m  - [pid=162] finished temporary directories cleanup[22m
+[2m  - [pid=162] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201157633Z-830580a6--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:57.700Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:57.734Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-4xVtlW --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=165
+[pid=165][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-4xVtlW --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=165[22m
+[2m  - [pid=165][err] error: Unable to allocate instance id[22m
+[2m  - [pid=165] &lt;gracefully close start&gt;[22m
+[2m  - [pid=165] &lt;kill&gt;[22m
+[2m  - [pid=165] &lt;will force kill&gt;[22m
+[2m  - [pid=165] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=165] starting temporary directories cleanup[22m
+[2m  - [pid=165] finished temporary directories cleanup[22m
+[2m  - [pid=165] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201157633Z-830580a6--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:57.738Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:11:57.773Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-MqCxRf --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=168
+[pid=168][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-MqCxRf --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=168[22m
+[2m  - [pid=168][err] error: Unable to allocate instance id[22m
+[2m  - [pid=168] &lt;gracefully close start&gt;[22m
+[2m  - [pid=168] &lt;kill&gt;[22m
+[2m  - [pid=168] &lt;will force kill&gt;[22m
+[2m  - [pid=168] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=168] starting temporary directories cleanup[22m
+[2m  - [pid=168] finished temporary directories cleanup[22m
+[2m  - [pid=168] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201209461Z-313fedb5</t>
+  </si>
+  <si>
+    <t>sim-20260913T201209461Z-313fedb5--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:12:09.465Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:12:09.523Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-UImGDj --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=63
+[pid=63][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-UImGDj --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=63[22m
+[2m  - [pid=63][err] error: Unable to allocate instance id[22m
+[2m  - [pid=63] &lt;gracefully close start&gt;[22m
+[2m  - [pid=63] &lt;kill&gt;[22m
+[2m  - [pid=63] &lt;will force kill&gt;[22m
+[2m  - [pid=63] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=63] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=63] starting temporary directories cleanup[22m
+[2m  - [pid=63] finished temporary directories cleanup[22m
+[2m  - [pid=63] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201214730Z-5e61a42f</t>
+  </si>
+  <si>
+    <t>sim-20260913T201214730Z-5e61a42f--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:12:14.734Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:12:14.790Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-Et49U8 --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=107
+[pid=107][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-Et49U8 --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=107[22m
+[2m  - [pid=107][err] error: Unable to allocate instance id[22m
+[2m  - [pid=107] &lt;gracefully close start&gt;[22m
+[2m  - [pid=107] &lt;kill&gt;[22m
+[2m  - [pid=107] &lt;will force kill&gt;[22m
+[2m  - [pid=107] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=107] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=107] starting temporary directories cleanup[22m
+[2m  - [pid=107] finished temporary directories cleanup[22m
+[2m  - [pid=107] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201220540Z-b469e637</t>
+  </si>
+  <si>
+    <t>sim-20260913T201220540Z-b469e637--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:12:20.544Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:12:20.610Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browserType.launch: Target page, context or browser has been closed
+Browser logs:
+&lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-wNlL1w --remote-debugging-pipe --no-startup-window
+&lt;launched&gt; pid=150
+[pid=150][err] error: Unable to allocate instance id
+Call log:
+[2m  - &lt;launching&gt; /var/lib/flatpak/exports/bin/com.google.Chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --headless --hide-scrollbars --mute-audio --blink-settings=primaryHoverType=2,availableHoverTypes=2,primaryPointerType=4,availablePointerTypes=4 --no-sandbox --no-first-run --no-default-browser-check --user-data-dir=/tmp/playwright_chromiumdev_profile-wNlL1w --remote-debugging-pipe --no-startup-window[22m
+[2m  - &lt;launched&gt; pid=150[22m
+[2m  - [pid=150][err] error: Unable to allocate instance id[22m
+[2m  - [pid=150] &lt;gracefully close start&gt;[22m
+[2m  - [pid=150] &lt;kill&gt;[22m
+[2m  - [pid=150] &lt;will force kill&gt;[22m
+[2m  - [pid=150] exception while trying to kill process: Error: kill ESRCH[22m
+[2m  - [pid=150] &lt;process did exit: exitCode=1, signal=null&gt;[22m
+[2m  - [pid=150] starting temporary directories cleanup[22m
+[2m  - [pid=150] finished temporary directories cleanup[22m
+[2m  - [pid=150] &lt;gracefully close end&gt;[22m
+</t>
+  </si>
+  <si>
+    <t>sim-20260913T201358619Z-6ed1592f</t>
+  </si>
+  <si>
+    <t>sim-20260913T201358619Z-6ed1592f--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>afb0ea1920b5edf535eadfba63719196c4ddd252</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:13:58.623Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:13:59.595Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: SecurityError: Failed to read the 'localStorage' property from 'Window': Access is denied for this document.
+    at UtilityScript.evaluate (&lt;anonymous&gt;:304:16)
+    at UtilityScript.&lt;anonymous&gt; (&lt;anonymous&gt;:1:44)</t>
+  </si>
+  <si>
+    <t>sim-20260913T201358619Z-6ed1592f--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:13:59.600Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:00.450Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201358619Z-6ed1592f--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:00.453Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:01.385Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201453101Z-6cf04497</t>
+  </si>
+  <si>
+    <t>sim-20260913T201453101Z-6cf04497--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:53.105Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:54.909Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201453101Z-6cf04497--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:54.916Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:57.195Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201453101Z-6cf04497--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:57.198Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:14:59.043Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201518390Z-79822fe2</t>
+  </si>
+  <si>
+    <t>sim-20260913T201518390Z-79822fe2--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:18.394Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:20.132Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201518390Z-79822fe2--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:20.138Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:22.488Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201518390Z-79822fe2--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:22.493Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:24.673Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201530833Z-36678337</t>
+  </si>
+  <si>
+    <t>sim-20260913T201530833Z-36678337--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:30.838Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:32.638Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201530833Z-36678337--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:32.647Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:35.221Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201530833Z-36678337--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:35.224Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:37.488Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201543873Z-428a550f</t>
+  </si>
+  <si>
+    <t>sim-20260913T201543873Z-428a550f--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:43.877Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:45.956Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201543873Z-428a550f--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:45.964Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:48.221Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201543873Z-428a550f--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:48.224Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:50.172Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201556691Z-37ebb9c9</t>
+  </si>
+  <si>
+    <t>sim-20260913T201556691Z-37ebb9c9--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:56.699Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:15:58.779Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201605085Z-3fd57e71</t>
+  </si>
+  <si>
+    <t>sim-20260913T201605085Z-3fd57e71--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:16:05.091Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:16:08.906Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T201614923Z-f9d0f9a0</t>
+  </si>
+  <si>
+    <t>sim-20260913T201614923Z-f9d0f9a0--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:16:14.928Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:16:16.883Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T202008684Z-ba615cf8</t>
+  </si>
+  <si>
+    <t>sim-20260913T202008684Z-ba615cf8--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:20:08.687Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:20:10.376Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T202008684Z-ba615cf8--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:20:10.380Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:20:12.540Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T202008684Z-ba615cf8--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:20:12.542Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:20:14.448Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T203754298Z-71feccb6</t>
+  </si>
+  <si>
+    <t>sim-20260913T203754298Z-71feccb6--ZUP-001-SENSE-SESSIO-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:37:54.303Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:37:56.356Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T203754298Z-71feccb6--ZUP-073-USER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:37:56.362Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:37:58.764Z</t>
+  </si>
+  <si>
+    <t>sim-20260913T203754298Z-71feccb6--ZUP-115-DEVELOPER-principal--a01</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:37:58.768Z</t>
+  </si>
+  <si>
+    <t>2026-09-13T20:38:01.142Z</t>
   </si>
 </sst>
 </file>
@@ -35836,7 +36635,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W33"/>
+  <dimension ref="A1:W75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -38197,6 +38996,2988 @@
         <v>825</v>
       </c>
     </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>946</v>
+      </c>
+      <c r="B34" t="s">
+        <v>947</v>
+      </c>
+      <c r="C34" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" t="s">
+        <v>56</v>
+      </c>
+      <c r="E34" t="s">
+        <v>61</v>
+      </c>
+      <c r="F34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G34" t="s">
+        <v>60</v>
+      </c>
+      <c r="H34" t="s">
+        <v>818</v>
+      </c>
+      <c r="I34" t="s">
+        <v>948</v>
+      </c>
+      <c r="J34" t="s">
+        <v>820</v>
+      </c>
+      <c r="K34" t="s">
+        <v>948</v>
+      </c>
+      <c r="L34" t="s">
+        <v>949</v>
+      </c>
+      <c r="M34" t="s">
+        <v>950</v>
+      </c>
+      <c r="N34">
+        <v>96</v>
+      </c>
+      <c r="O34">
+        <v>1</v>
+      </c>
+      <c r="P34" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>825</v>
+      </c>
+      <c r="R34" t="s">
+        <v>825</v>
+      </c>
+      <c r="S34" t="s">
+        <v>951</v>
+      </c>
+      <c r="T34" t="s">
+        <v>952</v>
+      </c>
+      <c r="U34" t="s">
+        <v>827</v>
+      </c>
+      <c r="V34" t="s">
+        <v>820</v>
+      </c>
+      <c r="W34" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>946</v>
+      </c>
+      <c r="B35" t="s">
+        <v>953</v>
+      </c>
+      <c r="C35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35" t="s">
+        <v>427</v>
+      </c>
+      <c r="E35" t="s">
+        <v>34</v>
+      </c>
+      <c r="F35" t="s">
+        <v>64</v>
+      </c>
+      <c r="G35" t="s">
+        <v>60</v>
+      </c>
+      <c r="H35" t="s">
+        <v>818</v>
+      </c>
+      <c r="I35" t="s">
+        <v>948</v>
+      </c>
+      <c r="J35" t="s">
+        <v>820</v>
+      </c>
+      <c r="K35" t="s">
+        <v>948</v>
+      </c>
+      <c r="L35" t="s">
+        <v>954</v>
+      </c>
+      <c r="M35" t="s">
+        <v>955</v>
+      </c>
+      <c r="N35">
+        <v>50</v>
+      </c>
+      <c r="O35">
+        <v>1</v>
+      </c>
+      <c r="P35" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>825</v>
+      </c>
+      <c r="R35" t="s">
+        <v>825</v>
+      </c>
+      <c r="S35" t="s">
+        <v>956</v>
+      </c>
+      <c r="T35" t="s">
+        <v>837</v>
+      </c>
+      <c r="U35" t="s">
+        <v>827</v>
+      </c>
+      <c r="V35" t="s">
+        <v>820</v>
+      </c>
+      <c r="W35" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>946</v>
+      </c>
+      <c r="B36" t="s">
+        <v>957</v>
+      </c>
+      <c r="C36" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" t="s">
+        <v>613</v>
+      </c>
+      <c r="E36" t="s">
+        <v>188</v>
+      </c>
+      <c r="F36" t="s">
+        <v>64</v>
+      </c>
+      <c r="G36" t="s">
+        <v>60</v>
+      </c>
+      <c r="H36" t="s">
+        <v>818</v>
+      </c>
+      <c r="I36" t="s">
+        <v>948</v>
+      </c>
+      <c r="J36" t="s">
+        <v>820</v>
+      </c>
+      <c r="K36" t="s">
+        <v>948</v>
+      </c>
+      <c r="L36" t="s">
+        <v>958</v>
+      </c>
+      <c r="M36" t="s">
+        <v>959</v>
+      </c>
+      <c r="N36">
+        <v>52</v>
+      </c>
+      <c r="O36">
+        <v>1</v>
+      </c>
+      <c r="P36" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>825</v>
+      </c>
+      <c r="R36" t="s">
+        <v>825</v>
+      </c>
+      <c r="S36" t="s">
+        <v>960</v>
+      </c>
+      <c r="T36" t="s">
+        <v>961</v>
+      </c>
+      <c r="U36" t="s">
+        <v>827</v>
+      </c>
+      <c r="V36" t="s">
+        <v>820</v>
+      </c>
+      <c r="W36" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>962</v>
+      </c>
+      <c r="B37" t="s">
+        <v>963</v>
+      </c>
+      <c r="C37" t="s">
+        <v>64</v>
+      </c>
+      <c r="D37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" t="s">
+        <v>61</v>
+      </c>
+      <c r="F37" t="s">
+        <v>64</v>
+      </c>
+      <c r="G37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H37" t="s">
+        <v>818</v>
+      </c>
+      <c r="I37" t="s">
+        <v>948</v>
+      </c>
+      <c r="J37" t="s">
+        <v>820</v>
+      </c>
+      <c r="K37" t="s">
+        <v>948</v>
+      </c>
+      <c r="L37" t="s">
+        <v>964</v>
+      </c>
+      <c r="M37" t="s">
+        <v>965</v>
+      </c>
+      <c r="N37">
+        <v>79</v>
+      </c>
+      <c r="O37">
+        <v>1</v>
+      </c>
+      <c r="P37" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>825</v>
+      </c>
+      <c r="R37" t="s">
+        <v>825</v>
+      </c>
+      <c r="S37" t="s">
+        <v>966</v>
+      </c>
+      <c r="T37" t="s">
+        <v>952</v>
+      </c>
+      <c r="U37" t="s">
+        <v>827</v>
+      </c>
+      <c r="V37" t="s">
+        <v>820</v>
+      </c>
+      <c r="W37" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>962</v>
+      </c>
+      <c r="B38" t="s">
+        <v>967</v>
+      </c>
+      <c r="C38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D38" t="s">
+        <v>427</v>
+      </c>
+      <c r="E38" t="s">
+        <v>34</v>
+      </c>
+      <c r="F38" t="s">
+        <v>64</v>
+      </c>
+      <c r="G38" t="s">
+        <v>60</v>
+      </c>
+      <c r="H38" t="s">
+        <v>818</v>
+      </c>
+      <c r="I38" t="s">
+        <v>948</v>
+      </c>
+      <c r="J38" t="s">
+        <v>820</v>
+      </c>
+      <c r="K38" t="s">
+        <v>948</v>
+      </c>
+      <c r="L38" t="s">
+        <v>968</v>
+      </c>
+      <c r="M38" t="s">
+        <v>969</v>
+      </c>
+      <c r="N38">
+        <v>57</v>
+      </c>
+      <c r="O38">
+        <v>1</v>
+      </c>
+      <c r="P38" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>825</v>
+      </c>
+      <c r="R38" t="s">
+        <v>825</v>
+      </c>
+      <c r="S38" t="s">
+        <v>970</v>
+      </c>
+      <c r="T38" t="s">
+        <v>837</v>
+      </c>
+      <c r="U38" t="s">
+        <v>827</v>
+      </c>
+      <c r="V38" t="s">
+        <v>820</v>
+      </c>
+      <c r="W38" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>962</v>
+      </c>
+      <c r="B39" t="s">
+        <v>971</v>
+      </c>
+      <c r="C39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D39" t="s">
+        <v>613</v>
+      </c>
+      <c r="E39" t="s">
+        <v>188</v>
+      </c>
+      <c r="F39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H39" t="s">
+        <v>818</v>
+      </c>
+      <c r="I39" t="s">
+        <v>948</v>
+      </c>
+      <c r="J39" t="s">
+        <v>820</v>
+      </c>
+      <c r="K39" t="s">
+        <v>948</v>
+      </c>
+      <c r="L39" t="s">
+        <v>972</v>
+      </c>
+      <c r="M39" t="s">
+        <v>973</v>
+      </c>
+      <c r="N39">
+        <v>55</v>
+      </c>
+      <c r="O39">
+        <v>1</v>
+      </c>
+      <c r="P39" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>825</v>
+      </c>
+      <c r="R39" t="s">
+        <v>825</v>
+      </c>
+      <c r="S39" t="s">
+        <v>974</v>
+      </c>
+      <c r="T39" t="s">
+        <v>961</v>
+      </c>
+      <c r="U39" t="s">
+        <v>827</v>
+      </c>
+      <c r="V39" t="s">
+        <v>820</v>
+      </c>
+      <c r="W39" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>975</v>
+      </c>
+      <c r="B40" t="s">
+        <v>976</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" t="s">
+        <v>61</v>
+      </c>
+      <c r="F40" t="s">
+        <v>64</v>
+      </c>
+      <c r="G40" t="s">
+        <v>60</v>
+      </c>
+      <c r="H40" t="s">
+        <v>818</v>
+      </c>
+      <c r="I40" t="s">
+        <v>948</v>
+      </c>
+      <c r="J40" t="s">
+        <v>820</v>
+      </c>
+      <c r="K40" t="s">
+        <v>948</v>
+      </c>
+      <c r="L40" t="s">
+        <v>977</v>
+      </c>
+      <c r="M40" t="s">
+        <v>978</v>
+      </c>
+      <c r="N40">
+        <v>57</v>
+      </c>
+      <c r="O40">
+        <v>1</v>
+      </c>
+      <c r="P40" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>825</v>
+      </c>
+      <c r="R40" t="s">
+        <v>825</v>
+      </c>
+      <c r="S40" t="s">
+        <v>979</v>
+      </c>
+      <c r="T40" t="s">
+        <v>952</v>
+      </c>
+      <c r="U40" t="s">
+        <v>827</v>
+      </c>
+      <c r="V40" t="s">
+        <v>820</v>
+      </c>
+      <c r="W40" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>975</v>
+      </c>
+      <c r="B41" t="s">
+        <v>980</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41" t="s">
+        <v>427</v>
+      </c>
+      <c r="E41" t="s">
+        <v>34</v>
+      </c>
+      <c r="F41" t="s">
+        <v>64</v>
+      </c>
+      <c r="G41" t="s">
+        <v>60</v>
+      </c>
+      <c r="H41" t="s">
+        <v>818</v>
+      </c>
+      <c r="I41" t="s">
+        <v>948</v>
+      </c>
+      <c r="J41" t="s">
+        <v>820</v>
+      </c>
+      <c r="K41" t="s">
+        <v>948</v>
+      </c>
+      <c r="L41" t="s">
+        <v>981</v>
+      </c>
+      <c r="M41" t="s">
+        <v>982</v>
+      </c>
+      <c r="N41">
+        <v>35</v>
+      </c>
+      <c r="O41">
+        <v>1</v>
+      </c>
+      <c r="P41" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>825</v>
+      </c>
+      <c r="R41" t="s">
+        <v>825</v>
+      </c>
+      <c r="S41" t="s">
+        <v>983</v>
+      </c>
+      <c r="T41" t="s">
+        <v>837</v>
+      </c>
+      <c r="U41" t="s">
+        <v>827</v>
+      </c>
+      <c r="V41" t="s">
+        <v>820</v>
+      </c>
+      <c r="W41" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>975</v>
+      </c>
+      <c r="B42" t="s">
+        <v>984</v>
+      </c>
+      <c r="C42" t="s">
+        <v>64</v>
+      </c>
+      <c r="D42" t="s">
+        <v>613</v>
+      </c>
+      <c r="E42" t="s">
+        <v>188</v>
+      </c>
+      <c r="F42" t="s">
+        <v>64</v>
+      </c>
+      <c r="G42" t="s">
+        <v>60</v>
+      </c>
+      <c r="H42" t="s">
+        <v>818</v>
+      </c>
+      <c r="I42" t="s">
+        <v>948</v>
+      </c>
+      <c r="J42" t="s">
+        <v>820</v>
+      </c>
+      <c r="K42" t="s">
+        <v>948</v>
+      </c>
+      <c r="L42" t="s">
+        <v>985</v>
+      </c>
+      <c r="M42" t="s">
+        <v>986</v>
+      </c>
+      <c r="N42">
+        <v>35</v>
+      </c>
+      <c r="O42">
+        <v>1</v>
+      </c>
+      <c r="P42" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>825</v>
+      </c>
+      <c r="R42" t="s">
+        <v>825</v>
+      </c>
+      <c r="S42" t="s">
+        <v>987</v>
+      </c>
+      <c r="T42" t="s">
+        <v>961</v>
+      </c>
+      <c r="U42" t="s">
+        <v>827</v>
+      </c>
+      <c r="V42" t="s">
+        <v>820</v>
+      </c>
+      <c r="W42" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>988</v>
+      </c>
+      <c r="B43" t="s">
+        <v>989</v>
+      </c>
+      <c r="C43" t="s">
+        <v>64</v>
+      </c>
+      <c r="D43" t="s">
+        <v>56</v>
+      </c>
+      <c r="E43" t="s">
+        <v>61</v>
+      </c>
+      <c r="F43" t="s">
+        <v>64</v>
+      </c>
+      <c r="G43" t="s">
+        <v>60</v>
+      </c>
+      <c r="H43" t="s">
+        <v>818</v>
+      </c>
+      <c r="I43" t="s">
+        <v>948</v>
+      </c>
+      <c r="J43" t="s">
+        <v>820</v>
+      </c>
+      <c r="K43" t="s">
+        <v>948</v>
+      </c>
+      <c r="L43" t="s">
+        <v>990</v>
+      </c>
+      <c r="M43" t="s">
+        <v>991</v>
+      </c>
+      <c r="N43">
+        <v>95</v>
+      </c>
+      <c r="O43">
+        <v>1</v>
+      </c>
+      <c r="P43" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>825</v>
+      </c>
+      <c r="R43" t="s">
+        <v>825</v>
+      </c>
+      <c r="S43" t="s">
+        <v>992</v>
+      </c>
+      <c r="T43" t="s">
+        <v>952</v>
+      </c>
+      <c r="U43" t="s">
+        <v>827</v>
+      </c>
+      <c r="V43" t="s">
+        <v>820</v>
+      </c>
+      <c r="W43" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>988</v>
+      </c>
+      <c r="B44" t="s">
+        <v>993</v>
+      </c>
+      <c r="C44" t="s">
+        <v>64</v>
+      </c>
+      <c r="D44" t="s">
+        <v>427</v>
+      </c>
+      <c r="E44" t="s">
+        <v>34</v>
+      </c>
+      <c r="F44" t="s">
+        <v>64</v>
+      </c>
+      <c r="G44" t="s">
+        <v>60</v>
+      </c>
+      <c r="H44" t="s">
+        <v>818</v>
+      </c>
+      <c r="I44" t="s">
+        <v>948</v>
+      </c>
+      <c r="J44" t="s">
+        <v>820</v>
+      </c>
+      <c r="K44" t="s">
+        <v>948</v>
+      </c>
+      <c r="L44" t="s">
+        <v>994</v>
+      </c>
+      <c r="M44" t="s">
+        <v>995</v>
+      </c>
+      <c r="N44">
+        <v>42</v>
+      </c>
+      <c r="O44">
+        <v>1</v>
+      </c>
+      <c r="P44" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>825</v>
+      </c>
+      <c r="R44" t="s">
+        <v>825</v>
+      </c>
+      <c r="S44" t="s">
+        <v>996</v>
+      </c>
+      <c r="T44" t="s">
+        <v>837</v>
+      </c>
+      <c r="U44" t="s">
+        <v>827</v>
+      </c>
+      <c r="V44" t="s">
+        <v>820</v>
+      </c>
+      <c r="W44" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>988</v>
+      </c>
+      <c r="B45" t="s">
+        <v>997</v>
+      </c>
+      <c r="C45" t="s">
+        <v>64</v>
+      </c>
+      <c r="D45" t="s">
+        <v>613</v>
+      </c>
+      <c r="E45" t="s">
+        <v>188</v>
+      </c>
+      <c r="F45" t="s">
+        <v>64</v>
+      </c>
+      <c r="G45" t="s">
+        <v>60</v>
+      </c>
+      <c r="H45" t="s">
+        <v>818</v>
+      </c>
+      <c r="I45" t="s">
+        <v>948</v>
+      </c>
+      <c r="J45" t="s">
+        <v>820</v>
+      </c>
+      <c r="K45" t="s">
+        <v>948</v>
+      </c>
+      <c r="L45" t="s">
+        <v>998</v>
+      </c>
+      <c r="M45" t="s">
+        <v>999</v>
+      </c>
+      <c r="N45">
+        <v>39</v>
+      </c>
+      <c r="O45">
+        <v>1</v>
+      </c>
+      <c r="P45" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>825</v>
+      </c>
+      <c r="R45" t="s">
+        <v>825</v>
+      </c>
+      <c r="S45" t="s">
+        <v>1000</v>
+      </c>
+      <c r="T45" t="s">
+        <v>961</v>
+      </c>
+      <c r="U45" t="s">
+        <v>827</v>
+      </c>
+      <c r="V45" t="s">
+        <v>820</v>
+      </c>
+      <c r="W45" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C46" t="s">
+        <v>64</v>
+      </c>
+      <c r="D46" t="s">
+        <v>56</v>
+      </c>
+      <c r="E46" t="s">
+        <v>61</v>
+      </c>
+      <c r="F46" t="s">
+        <v>64</v>
+      </c>
+      <c r="G46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H46" t="s">
+        <v>818</v>
+      </c>
+      <c r="I46" t="s">
+        <v>948</v>
+      </c>
+      <c r="J46" t="s">
+        <v>820</v>
+      </c>
+      <c r="K46" t="s">
+        <v>948</v>
+      </c>
+      <c r="L46" t="s">
+        <v>1003</v>
+      </c>
+      <c r="M46" t="s">
+        <v>1004</v>
+      </c>
+      <c r="N46">
+        <v>57</v>
+      </c>
+      <c r="O46">
+        <v>1</v>
+      </c>
+      <c r="P46" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>825</v>
+      </c>
+      <c r="R46" t="s">
+        <v>825</v>
+      </c>
+      <c r="S46" t="s">
+        <v>1005</v>
+      </c>
+      <c r="T46" t="s">
+        <v>952</v>
+      </c>
+      <c r="U46" t="s">
+        <v>827</v>
+      </c>
+      <c r="V46" t="s">
+        <v>820</v>
+      </c>
+      <c r="W46" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C47" t="s">
+        <v>64</v>
+      </c>
+      <c r="D47" t="s">
+        <v>427</v>
+      </c>
+      <c r="E47" t="s">
+        <v>34</v>
+      </c>
+      <c r="F47" t="s">
+        <v>64</v>
+      </c>
+      <c r="G47" t="s">
+        <v>60</v>
+      </c>
+      <c r="H47" t="s">
+        <v>818</v>
+      </c>
+      <c r="I47" t="s">
+        <v>948</v>
+      </c>
+      <c r="J47" t="s">
+        <v>820</v>
+      </c>
+      <c r="K47" t="s">
+        <v>948</v>
+      </c>
+      <c r="L47" t="s">
+        <v>1007</v>
+      </c>
+      <c r="M47" t="s">
+        <v>1008</v>
+      </c>
+      <c r="N47">
+        <v>34</v>
+      </c>
+      <c r="O47">
+        <v>1</v>
+      </c>
+      <c r="P47" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>825</v>
+      </c>
+      <c r="R47" t="s">
+        <v>825</v>
+      </c>
+      <c r="S47" t="s">
+        <v>1009</v>
+      </c>
+      <c r="T47" t="s">
+        <v>837</v>
+      </c>
+      <c r="U47" t="s">
+        <v>827</v>
+      </c>
+      <c r="V47" t="s">
+        <v>820</v>
+      </c>
+      <c r="W47" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1010</v>
+      </c>
+      <c r="C48" t="s">
+        <v>64</v>
+      </c>
+      <c r="D48" t="s">
+        <v>613</v>
+      </c>
+      <c r="E48" t="s">
+        <v>188</v>
+      </c>
+      <c r="F48" t="s">
+        <v>64</v>
+      </c>
+      <c r="G48" t="s">
+        <v>60</v>
+      </c>
+      <c r="H48" t="s">
+        <v>818</v>
+      </c>
+      <c r="I48" t="s">
+        <v>948</v>
+      </c>
+      <c r="J48" t="s">
+        <v>820</v>
+      </c>
+      <c r="K48" t="s">
+        <v>948</v>
+      </c>
+      <c r="L48" t="s">
+        <v>1011</v>
+      </c>
+      <c r="M48" t="s">
+        <v>1012</v>
+      </c>
+      <c r="N48">
+        <v>35</v>
+      </c>
+      <c r="O48">
+        <v>1</v>
+      </c>
+      <c r="P48" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>825</v>
+      </c>
+      <c r="R48" t="s">
+        <v>825</v>
+      </c>
+      <c r="S48" t="s">
+        <v>1013</v>
+      </c>
+      <c r="T48" t="s">
+        <v>961</v>
+      </c>
+      <c r="U48" t="s">
+        <v>827</v>
+      </c>
+      <c r="V48" t="s">
+        <v>820</v>
+      </c>
+      <c r="W48" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C49" t="s">
+        <v>64</v>
+      </c>
+      <c r="D49" t="s">
+        <v>613</v>
+      </c>
+      <c r="E49" t="s">
+        <v>188</v>
+      </c>
+      <c r="F49" t="s">
+        <v>64</v>
+      </c>
+      <c r="G49" t="s">
+        <v>60</v>
+      </c>
+      <c r="H49" t="s">
+        <v>818</v>
+      </c>
+      <c r="I49" t="s">
+        <v>948</v>
+      </c>
+      <c r="J49" t="s">
+        <v>820</v>
+      </c>
+      <c r="K49" t="s">
+        <v>948</v>
+      </c>
+      <c r="L49" t="s">
+        <v>1016</v>
+      </c>
+      <c r="M49" t="s">
+        <v>1017</v>
+      </c>
+      <c r="N49">
+        <v>58</v>
+      </c>
+      <c r="O49">
+        <v>1</v>
+      </c>
+      <c r="P49" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>825</v>
+      </c>
+      <c r="R49" t="s">
+        <v>825</v>
+      </c>
+      <c r="S49" t="s">
+        <v>1018</v>
+      </c>
+      <c r="T49" t="s">
+        <v>961</v>
+      </c>
+      <c r="U49" t="s">
+        <v>827</v>
+      </c>
+      <c r="V49" t="s">
+        <v>820</v>
+      </c>
+      <c r="W49" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B50" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C50" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" t="s">
+        <v>427</v>
+      </c>
+      <c r="E50" t="s">
+        <v>34</v>
+      </c>
+      <c r="F50" t="s">
+        <v>64</v>
+      </c>
+      <c r="G50" t="s">
+        <v>60</v>
+      </c>
+      <c r="H50" t="s">
+        <v>818</v>
+      </c>
+      <c r="I50" t="s">
+        <v>948</v>
+      </c>
+      <c r="J50" t="s">
+        <v>820</v>
+      </c>
+      <c r="K50" t="s">
+        <v>948</v>
+      </c>
+      <c r="L50" t="s">
+        <v>1021</v>
+      </c>
+      <c r="M50" t="s">
+        <v>1022</v>
+      </c>
+      <c r="N50">
+        <v>56</v>
+      </c>
+      <c r="O50">
+        <v>1</v>
+      </c>
+      <c r="P50" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>825</v>
+      </c>
+      <c r="R50" t="s">
+        <v>825</v>
+      </c>
+      <c r="S50" t="s">
+        <v>1023</v>
+      </c>
+      <c r="T50" t="s">
+        <v>837</v>
+      </c>
+      <c r="U50" t="s">
+        <v>827</v>
+      </c>
+      <c r="V50" t="s">
+        <v>820</v>
+      </c>
+      <c r="W50" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B51" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C51" t="s">
+        <v>64</v>
+      </c>
+      <c r="D51" t="s">
+        <v>56</v>
+      </c>
+      <c r="E51" t="s">
+        <v>61</v>
+      </c>
+      <c r="F51" t="s">
+        <v>64</v>
+      </c>
+      <c r="G51" t="s">
+        <v>60</v>
+      </c>
+      <c r="H51" t="s">
+        <v>818</v>
+      </c>
+      <c r="I51" t="s">
+        <v>948</v>
+      </c>
+      <c r="J51" t="s">
+        <v>820</v>
+      </c>
+      <c r="K51" t="s">
+        <v>948</v>
+      </c>
+      <c r="L51" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M51" t="s">
+        <v>1027</v>
+      </c>
+      <c r="N51">
+        <v>66</v>
+      </c>
+      <c r="O51">
+        <v>1</v>
+      </c>
+      <c r="P51" t="s">
+        <v>891</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>825</v>
+      </c>
+      <c r="R51" t="s">
+        <v>825</v>
+      </c>
+      <c r="S51" t="s">
+        <v>1028</v>
+      </c>
+      <c r="T51" t="s">
+        <v>952</v>
+      </c>
+      <c r="U51" t="s">
+        <v>827</v>
+      </c>
+      <c r="V51" t="s">
+        <v>820</v>
+      </c>
+      <c r="W51" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52" t="s">
+        <v>56</v>
+      </c>
+      <c r="E52" t="s">
+        <v>61</v>
+      </c>
+      <c r="F52" t="s">
+        <v>64</v>
+      </c>
+      <c r="G52" t="s">
+        <v>60</v>
+      </c>
+      <c r="H52" t="s">
+        <v>818</v>
+      </c>
+      <c r="I52" t="s">
+        <v>819</v>
+      </c>
+      <c r="J52" t="s">
+        <v>820</v>
+      </c>
+      <c r="K52" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L52" t="s">
+        <v>1032</v>
+      </c>
+      <c r="M52" t="s">
+        <v>1033</v>
+      </c>
+      <c r="N52">
+        <v>972</v>
+      </c>
+      <c r="O52">
+        <v>1</v>
+      </c>
+      <c r="P52" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>825</v>
+      </c>
+      <c r="R52" t="s">
+        <v>825</v>
+      </c>
+      <c r="S52" t="s">
+        <v>1034</v>
+      </c>
+      <c r="T52" t="s">
+        <v>952</v>
+      </c>
+      <c r="U52" t="s">
+        <v>827</v>
+      </c>
+      <c r="V52" t="s">
+        <v>820</v>
+      </c>
+      <c r="W52" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53" t="s">
+        <v>427</v>
+      </c>
+      <c r="E53" t="s">
+        <v>34</v>
+      </c>
+      <c r="F53" t="s">
+        <v>64</v>
+      </c>
+      <c r="G53" t="s">
+        <v>60</v>
+      </c>
+      <c r="H53" t="s">
+        <v>818</v>
+      </c>
+      <c r="I53" t="s">
+        <v>819</v>
+      </c>
+      <c r="J53" t="s">
+        <v>820</v>
+      </c>
+      <c r="K53" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L53" t="s">
+        <v>1036</v>
+      </c>
+      <c r="M53" t="s">
+        <v>1037</v>
+      </c>
+      <c r="N53">
+        <v>850</v>
+      </c>
+      <c r="O53">
+        <v>1</v>
+      </c>
+      <c r="P53" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>825</v>
+      </c>
+      <c r="R53" t="s">
+        <v>825</v>
+      </c>
+      <c r="S53" t="s">
+        <v>1034</v>
+      </c>
+      <c r="T53" t="s">
+        <v>837</v>
+      </c>
+      <c r="U53" t="s">
+        <v>827</v>
+      </c>
+      <c r="V53" t="s">
+        <v>820</v>
+      </c>
+      <c r="W53" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C54" t="s">
+        <v>64</v>
+      </c>
+      <c r="D54" t="s">
+        <v>613</v>
+      </c>
+      <c r="E54" t="s">
+        <v>188</v>
+      </c>
+      <c r="F54" t="s">
+        <v>64</v>
+      </c>
+      <c r="G54" t="s">
+        <v>60</v>
+      </c>
+      <c r="H54" t="s">
+        <v>818</v>
+      </c>
+      <c r="I54" t="s">
+        <v>819</v>
+      </c>
+      <c r="J54" t="s">
+        <v>820</v>
+      </c>
+      <c r="K54" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L54" t="s">
+        <v>1039</v>
+      </c>
+      <c r="M54" t="s">
+        <v>1040</v>
+      </c>
+      <c r="N54">
+        <v>932</v>
+      </c>
+      <c r="O54">
+        <v>1</v>
+      </c>
+      <c r="P54" t="s">
+        <v>835</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>825</v>
+      </c>
+      <c r="R54" t="s">
+        <v>825</v>
+      </c>
+      <c r="S54" t="s">
+        <v>1034</v>
+      </c>
+      <c r="T54" t="s">
+        <v>961</v>
+      </c>
+      <c r="U54" t="s">
+        <v>827</v>
+      </c>
+      <c r="V54" t="s">
+        <v>820</v>
+      </c>
+      <c r="W54" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C55" t="s">
+        <v>64</v>
+      </c>
+      <c r="D55" t="s">
+        <v>56</v>
+      </c>
+      <c r="E55" t="s">
+        <v>61</v>
+      </c>
+      <c r="F55" t="s">
+        <v>64</v>
+      </c>
+      <c r="G55" t="s">
+        <v>60</v>
+      </c>
+      <c r="H55" t="s">
+        <v>818</v>
+      </c>
+      <c r="I55" t="s">
+        <v>819</v>
+      </c>
+      <c r="J55" t="s">
+        <v>820</v>
+      </c>
+      <c r="K55" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L55" t="s">
+        <v>1043</v>
+      </c>
+      <c r="M55" t="s">
+        <v>1044</v>
+      </c>
+      <c r="N55">
+        <v>1804</v>
+      </c>
+      <c r="O55">
+        <v>1</v>
+      </c>
+      <c r="P55" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>825</v>
+      </c>
+      <c r="R55" t="s">
+        <v>825</v>
+      </c>
+      <c r="S55" t="s">
+        <v>826</v>
+      </c>
+      <c r="T55" t="s">
+        <v>825</v>
+      </c>
+      <c r="U55" t="s">
+        <v>827</v>
+      </c>
+      <c r="V55" t="s">
+        <v>820</v>
+      </c>
+      <c r="W55" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C56" t="s">
+        <v>64</v>
+      </c>
+      <c r="D56" t="s">
+        <v>427</v>
+      </c>
+      <c r="E56" t="s">
+        <v>34</v>
+      </c>
+      <c r="F56" t="s">
+        <v>64</v>
+      </c>
+      <c r="G56" t="s">
+        <v>60</v>
+      </c>
+      <c r="H56" t="s">
+        <v>818</v>
+      </c>
+      <c r="I56" t="s">
+        <v>819</v>
+      </c>
+      <c r="J56" t="s">
+        <v>820</v>
+      </c>
+      <c r="K56" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L56" t="s">
+        <v>1046</v>
+      </c>
+      <c r="M56" t="s">
+        <v>1047</v>
+      </c>
+      <c r="N56">
+        <v>2279</v>
+      </c>
+      <c r="O56">
+        <v>1</v>
+      </c>
+      <c r="P56" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>825</v>
+      </c>
+      <c r="R56" t="s">
+        <v>825</v>
+      </c>
+      <c r="S56" t="s">
+        <v>826</v>
+      </c>
+      <c r="T56" t="s">
+        <v>825</v>
+      </c>
+      <c r="U56" t="s">
+        <v>827</v>
+      </c>
+      <c r="V56" t="s">
+        <v>820</v>
+      </c>
+      <c r="W56" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B57" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C57" t="s">
+        <v>64</v>
+      </c>
+      <c r="D57" t="s">
+        <v>613</v>
+      </c>
+      <c r="E57" t="s">
+        <v>188</v>
+      </c>
+      <c r="F57" t="s">
+        <v>64</v>
+      </c>
+      <c r="G57" t="s">
+        <v>60</v>
+      </c>
+      <c r="H57" t="s">
+        <v>818</v>
+      </c>
+      <c r="I57" t="s">
+        <v>819</v>
+      </c>
+      <c r="J57" t="s">
+        <v>820</v>
+      </c>
+      <c r="K57" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L57" t="s">
+        <v>1049</v>
+      </c>
+      <c r="M57" t="s">
+        <v>1050</v>
+      </c>
+      <c r="N57">
+        <v>1845</v>
+      </c>
+      <c r="O57">
+        <v>1</v>
+      </c>
+      <c r="P57" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>825</v>
+      </c>
+      <c r="R57" t="s">
+        <v>825</v>
+      </c>
+      <c r="S57" t="s">
+        <v>826</v>
+      </c>
+      <c r="T57" t="s">
+        <v>825</v>
+      </c>
+      <c r="U57" t="s">
+        <v>827</v>
+      </c>
+      <c r="V57" t="s">
+        <v>820</v>
+      </c>
+      <c r="W57" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C58" t="s">
+        <v>64</v>
+      </c>
+      <c r="D58" t="s">
+        <v>56</v>
+      </c>
+      <c r="E58" t="s">
+        <v>61</v>
+      </c>
+      <c r="F58" t="s">
+        <v>64</v>
+      </c>
+      <c r="G58" t="s">
+        <v>60</v>
+      </c>
+      <c r="H58" t="s">
+        <v>818</v>
+      </c>
+      <c r="I58" t="s">
+        <v>819</v>
+      </c>
+      <c r="J58" t="s">
+        <v>820</v>
+      </c>
+      <c r="K58" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L58" t="s">
+        <v>1053</v>
+      </c>
+      <c r="M58" t="s">
+        <v>1054</v>
+      </c>
+      <c r="N58">
+        <v>1738</v>
+      </c>
+      <c r="O58">
+        <v>1</v>
+      </c>
+      <c r="P58" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>825</v>
+      </c>
+      <c r="R58" t="s">
+        <v>825</v>
+      </c>
+      <c r="S58" t="s">
+        <v>826</v>
+      </c>
+      <c r="T58" t="s">
+        <v>825</v>
+      </c>
+      <c r="U58" t="s">
+        <v>827</v>
+      </c>
+      <c r="V58" t="s">
+        <v>820</v>
+      </c>
+      <c r="W58" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C59" t="s">
+        <v>64</v>
+      </c>
+      <c r="D59" t="s">
+        <v>427</v>
+      </c>
+      <c r="E59" t="s">
+        <v>34</v>
+      </c>
+      <c r="F59" t="s">
+        <v>64</v>
+      </c>
+      <c r="G59" t="s">
+        <v>60</v>
+      </c>
+      <c r="H59" t="s">
+        <v>818</v>
+      </c>
+      <c r="I59" t="s">
+        <v>819</v>
+      </c>
+      <c r="J59" t="s">
+        <v>820</v>
+      </c>
+      <c r="K59" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L59" t="s">
+        <v>1056</v>
+      </c>
+      <c r="M59" t="s">
+        <v>1057</v>
+      </c>
+      <c r="N59">
+        <v>2350</v>
+      </c>
+      <c r="O59">
+        <v>1</v>
+      </c>
+      <c r="P59" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>825</v>
+      </c>
+      <c r="R59" t="s">
+        <v>825</v>
+      </c>
+      <c r="S59" t="s">
+        <v>826</v>
+      </c>
+      <c r="T59" t="s">
+        <v>825</v>
+      </c>
+      <c r="U59" t="s">
+        <v>827</v>
+      </c>
+      <c r="V59" t="s">
+        <v>820</v>
+      </c>
+      <c r="W59" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B60" t="s">
+        <v>1058</v>
+      </c>
+      <c r="C60" t="s">
+        <v>64</v>
+      </c>
+      <c r="D60" t="s">
+        <v>613</v>
+      </c>
+      <c r="E60" t="s">
+        <v>188</v>
+      </c>
+      <c r="F60" t="s">
+        <v>64</v>
+      </c>
+      <c r="G60" t="s">
+        <v>60</v>
+      </c>
+      <c r="H60" t="s">
+        <v>818</v>
+      </c>
+      <c r="I60" t="s">
+        <v>819</v>
+      </c>
+      <c r="J60" t="s">
+        <v>820</v>
+      </c>
+      <c r="K60" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L60" t="s">
+        <v>1059</v>
+      </c>
+      <c r="M60" t="s">
+        <v>1060</v>
+      </c>
+      <c r="N60">
+        <v>2180</v>
+      </c>
+      <c r="O60">
+        <v>1</v>
+      </c>
+      <c r="P60" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>825</v>
+      </c>
+      <c r="R60" t="s">
+        <v>825</v>
+      </c>
+      <c r="S60" t="s">
+        <v>826</v>
+      </c>
+      <c r="T60" t="s">
+        <v>825</v>
+      </c>
+      <c r="U60" t="s">
+        <v>827</v>
+      </c>
+      <c r="V60" t="s">
+        <v>820</v>
+      </c>
+      <c r="W60" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B61" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C61" t="s">
+        <v>64</v>
+      </c>
+      <c r="D61" t="s">
+        <v>56</v>
+      </c>
+      <c r="E61" t="s">
+        <v>61</v>
+      </c>
+      <c r="F61" t="s">
+        <v>64</v>
+      </c>
+      <c r="G61" t="s">
+        <v>60</v>
+      </c>
+      <c r="H61" t="s">
+        <v>818</v>
+      </c>
+      <c r="I61" t="s">
+        <v>819</v>
+      </c>
+      <c r="J61" t="s">
+        <v>820</v>
+      </c>
+      <c r="K61" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L61" t="s">
+        <v>1063</v>
+      </c>
+      <c r="M61" t="s">
+        <v>1064</v>
+      </c>
+      <c r="N61">
+        <v>1800</v>
+      </c>
+      <c r="O61">
+        <v>1</v>
+      </c>
+      <c r="P61" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>825</v>
+      </c>
+      <c r="R61" t="s">
+        <v>825</v>
+      </c>
+      <c r="S61" t="s">
+        <v>826</v>
+      </c>
+      <c r="T61" t="s">
+        <v>825</v>
+      </c>
+      <c r="U61" t="s">
+        <v>827</v>
+      </c>
+      <c r="V61" t="s">
+        <v>820</v>
+      </c>
+      <c r="W61" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B62" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C62" t="s">
+        <v>64</v>
+      </c>
+      <c r="D62" t="s">
+        <v>427</v>
+      </c>
+      <c r="E62" t="s">
+        <v>34</v>
+      </c>
+      <c r="F62" t="s">
+        <v>64</v>
+      </c>
+      <c r="G62" t="s">
+        <v>60</v>
+      </c>
+      <c r="H62" t="s">
+        <v>818</v>
+      </c>
+      <c r="I62" t="s">
+        <v>819</v>
+      </c>
+      <c r="J62" t="s">
+        <v>820</v>
+      </c>
+      <c r="K62" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L62" t="s">
+        <v>1066</v>
+      </c>
+      <c r="M62" t="s">
+        <v>1067</v>
+      </c>
+      <c r="N62">
+        <v>2574</v>
+      </c>
+      <c r="O62">
+        <v>1</v>
+      </c>
+      <c r="P62" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q62" t="s">
+        <v>825</v>
+      </c>
+      <c r="R62" t="s">
+        <v>825</v>
+      </c>
+      <c r="S62" t="s">
+        <v>826</v>
+      </c>
+      <c r="T62" t="s">
+        <v>825</v>
+      </c>
+      <c r="U62" t="s">
+        <v>827</v>
+      </c>
+      <c r="V62" t="s">
+        <v>820</v>
+      </c>
+      <c r="W62" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B63" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C63" t="s">
+        <v>64</v>
+      </c>
+      <c r="D63" t="s">
+        <v>613</v>
+      </c>
+      <c r="E63" t="s">
+        <v>188</v>
+      </c>
+      <c r="F63" t="s">
+        <v>64</v>
+      </c>
+      <c r="G63" t="s">
+        <v>60</v>
+      </c>
+      <c r="H63" t="s">
+        <v>818</v>
+      </c>
+      <c r="I63" t="s">
+        <v>819</v>
+      </c>
+      <c r="J63" t="s">
+        <v>820</v>
+      </c>
+      <c r="K63" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L63" t="s">
+        <v>1069</v>
+      </c>
+      <c r="M63" t="s">
+        <v>1070</v>
+      </c>
+      <c r="N63">
+        <v>2264</v>
+      </c>
+      <c r="O63">
+        <v>1</v>
+      </c>
+      <c r="P63" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>825</v>
+      </c>
+      <c r="R63" t="s">
+        <v>825</v>
+      </c>
+      <c r="S63" t="s">
+        <v>826</v>
+      </c>
+      <c r="T63" t="s">
+        <v>825</v>
+      </c>
+      <c r="U63" t="s">
+        <v>827</v>
+      </c>
+      <c r="V63" t="s">
+        <v>820</v>
+      </c>
+      <c r="W63" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B64" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C64" t="s">
+        <v>64</v>
+      </c>
+      <c r="D64" t="s">
+        <v>56</v>
+      </c>
+      <c r="E64" t="s">
+        <v>61</v>
+      </c>
+      <c r="F64" t="s">
+        <v>64</v>
+      </c>
+      <c r="G64" t="s">
+        <v>60</v>
+      </c>
+      <c r="H64" t="s">
+        <v>818</v>
+      </c>
+      <c r="I64" t="s">
+        <v>819</v>
+      </c>
+      <c r="J64" t="s">
+        <v>820</v>
+      </c>
+      <c r="K64" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L64" t="s">
+        <v>1073</v>
+      </c>
+      <c r="M64" t="s">
+        <v>1074</v>
+      </c>
+      <c r="N64">
+        <v>2079</v>
+      </c>
+      <c r="O64">
+        <v>1</v>
+      </c>
+      <c r="P64" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>825</v>
+      </c>
+      <c r="R64" t="s">
+        <v>825</v>
+      </c>
+      <c r="S64" t="s">
+        <v>826</v>
+      </c>
+      <c r="T64" t="s">
+        <v>825</v>
+      </c>
+      <c r="U64" t="s">
+        <v>827</v>
+      </c>
+      <c r="V64" t="s">
+        <v>820</v>
+      </c>
+      <c r="W64" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B65" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C65" t="s">
+        <v>64</v>
+      </c>
+      <c r="D65" t="s">
+        <v>427</v>
+      </c>
+      <c r="E65" t="s">
+        <v>34</v>
+      </c>
+      <c r="F65" t="s">
+        <v>64</v>
+      </c>
+      <c r="G65" t="s">
+        <v>60</v>
+      </c>
+      <c r="H65" t="s">
+        <v>818</v>
+      </c>
+      <c r="I65" t="s">
+        <v>819</v>
+      </c>
+      <c r="J65" t="s">
+        <v>820</v>
+      </c>
+      <c r="K65" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L65" t="s">
+        <v>1076</v>
+      </c>
+      <c r="M65" t="s">
+        <v>1077</v>
+      </c>
+      <c r="N65">
+        <v>2257</v>
+      </c>
+      <c r="O65">
+        <v>1</v>
+      </c>
+      <c r="P65" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>825</v>
+      </c>
+      <c r="R65" t="s">
+        <v>825</v>
+      </c>
+      <c r="S65" t="s">
+        <v>826</v>
+      </c>
+      <c r="T65" t="s">
+        <v>825</v>
+      </c>
+      <c r="U65" t="s">
+        <v>827</v>
+      </c>
+      <c r="V65" t="s">
+        <v>820</v>
+      </c>
+      <c r="W65" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B66" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C66" t="s">
+        <v>64</v>
+      </c>
+      <c r="D66" t="s">
+        <v>613</v>
+      </c>
+      <c r="E66" t="s">
+        <v>188</v>
+      </c>
+      <c r="F66" t="s">
+        <v>64</v>
+      </c>
+      <c r="G66" t="s">
+        <v>60</v>
+      </c>
+      <c r="H66" t="s">
+        <v>818</v>
+      </c>
+      <c r="I66" t="s">
+        <v>819</v>
+      </c>
+      <c r="J66" t="s">
+        <v>820</v>
+      </c>
+      <c r="K66" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L66" t="s">
+        <v>1079</v>
+      </c>
+      <c r="M66" t="s">
+        <v>1080</v>
+      </c>
+      <c r="N66">
+        <v>1948</v>
+      </c>
+      <c r="O66">
+        <v>1</v>
+      </c>
+      <c r="P66" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>825</v>
+      </c>
+      <c r="R66" t="s">
+        <v>825</v>
+      </c>
+      <c r="S66" t="s">
+        <v>826</v>
+      </c>
+      <c r="T66" t="s">
+        <v>825</v>
+      </c>
+      <c r="U66" t="s">
+        <v>827</v>
+      </c>
+      <c r="V66" t="s">
+        <v>820</v>
+      </c>
+      <c r="W66" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B67" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C67" t="s">
+        <v>64</v>
+      </c>
+      <c r="D67" t="s">
+        <v>613</v>
+      </c>
+      <c r="E67" t="s">
+        <v>188</v>
+      </c>
+      <c r="F67" t="s">
+        <v>64</v>
+      </c>
+      <c r="G67" t="s">
+        <v>60</v>
+      </c>
+      <c r="H67" t="s">
+        <v>818</v>
+      </c>
+      <c r="I67" t="s">
+        <v>819</v>
+      </c>
+      <c r="J67" t="s">
+        <v>820</v>
+      </c>
+      <c r="K67" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L67" t="s">
+        <v>1083</v>
+      </c>
+      <c r="M67" t="s">
+        <v>1084</v>
+      </c>
+      <c r="N67">
+        <v>2080</v>
+      </c>
+      <c r="O67">
+        <v>1</v>
+      </c>
+      <c r="P67" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>825</v>
+      </c>
+      <c r="R67" t="s">
+        <v>825</v>
+      </c>
+      <c r="S67" t="s">
+        <v>826</v>
+      </c>
+      <c r="T67" t="s">
+        <v>825</v>
+      </c>
+      <c r="U67" t="s">
+        <v>827</v>
+      </c>
+      <c r="V67" t="s">
+        <v>820</v>
+      </c>
+      <c r="W67" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B68" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C68" t="s">
+        <v>64</v>
+      </c>
+      <c r="D68" t="s">
+        <v>427</v>
+      </c>
+      <c r="E68" t="s">
+        <v>34</v>
+      </c>
+      <c r="F68" t="s">
+        <v>64</v>
+      </c>
+      <c r="G68" t="s">
+        <v>60</v>
+      </c>
+      <c r="H68" t="s">
+        <v>818</v>
+      </c>
+      <c r="I68" t="s">
+        <v>819</v>
+      </c>
+      <c r="J68" t="s">
+        <v>820</v>
+      </c>
+      <c r="K68" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L68" t="s">
+        <v>1087</v>
+      </c>
+      <c r="M68" t="s">
+        <v>1088</v>
+      </c>
+      <c r="N68">
+        <v>3815</v>
+      </c>
+      <c r="O68">
+        <v>1</v>
+      </c>
+      <c r="P68" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>825</v>
+      </c>
+      <c r="R68" t="s">
+        <v>825</v>
+      </c>
+      <c r="S68" t="s">
+        <v>826</v>
+      </c>
+      <c r="T68" t="s">
+        <v>825</v>
+      </c>
+      <c r="U68" t="s">
+        <v>827</v>
+      </c>
+      <c r="V68" t="s">
+        <v>820</v>
+      </c>
+      <c r="W68" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B69" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C69" t="s">
+        <v>64</v>
+      </c>
+      <c r="D69" t="s">
+        <v>56</v>
+      </c>
+      <c r="E69" t="s">
+        <v>61</v>
+      </c>
+      <c r="F69" t="s">
+        <v>64</v>
+      </c>
+      <c r="G69" t="s">
+        <v>60</v>
+      </c>
+      <c r="H69" t="s">
+        <v>818</v>
+      </c>
+      <c r="I69" t="s">
+        <v>819</v>
+      </c>
+      <c r="J69" t="s">
+        <v>820</v>
+      </c>
+      <c r="K69" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L69" t="s">
+        <v>1091</v>
+      </c>
+      <c r="M69" t="s">
+        <v>1092</v>
+      </c>
+      <c r="N69">
+        <v>1955</v>
+      </c>
+      <c r="O69">
+        <v>1</v>
+      </c>
+      <c r="P69" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>825</v>
+      </c>
+      <c r="R69" t="s">
+        <v>825</v>
+      </c>
+      <c r="S69" t="s">
+        <v>826</v>
+      </c>
+      <c r="T69" t="s">
+        <v>825</v>
+      </c>
+      <c r="U69" t="s">
+        <v>827</v>
+      </c>
+      <c r="V69" t="s">
+        <v>820</v>
+      </c>
+      <c r="W69" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B70" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C70" t="s">
+        <v>64</v>
+      </c>
+      <c r="D70" t="s">
+        <v>56</v>
+      </c>
+      <c r="E70" t="s">
+        <v>61</v>
+      </c>
+      <c r="F70" t="s">
+        <v>64</v>
+      </c>
+      <c r="G70" t="s">
+        <v>60</v>
+      </c>
+      <c r="H70" t="s">
+        <v>818</v>
+      </c>
+      <c r="I70" t="s">
+        <v>819</v>
+      </c>
+      <c r="J70" t="s">
+        <v>820</v>
+      </c>
+      <c r="K70" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L70" t="s">
+        <v>1095</v>
+      </c>
+      <c r="M70" t="s">
+        <v>1096</v>
+      </c>
+      <c r="N70">
+        <v>1689</v>
+      </c>
+      <c r="O70">
+        <v>1</v>
+      </c>
+      <c r="P70" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>825</v>
+      </c>
+      <c r="R70" t="s">
+        <v>825</v>
+      </c>
+      <c r="S70" t="s">
+        <v>826</v>
+      </c>
+      <c r="T70" t="s">
+        <v>825</v>
+      </c>
+      <c r="U70" t="s">
+        <v>827</v>
+      </c>
+      <c r="V70" t="s">
+        <v>820</v>
+      </c>
+      <c r="W70" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B71" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C71" t="s">
+        <v>64</v>
+      </c>
+      <c r="D71" t="s">
+        <v>427</v>
+      </c>
+      <c r="E71" t="s">
+        <v>34</v>
+      </c>
+      <c r="F71" t="s">
+        <v>64</v>
+      </c>
+      <c r="G71" t="s">
+        <v>60</v>
+      </c>
+      <c r="H71" t="s">
+        <v>818</v>
+      </c>
+      <c r="I71" t="s">
+        <v>819</v>
+      </c>
+      <c r="J71" t="s">
+        <v>820</v>
+      </c>
+      <c r="K71" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L71" t="s">
+        <v>1098</v>
+      </c>
+      <c r="M71" t="s">
+        <v>1099</v>
+      </c>
+      <c r="N71">
+        <v>2160</v>
+      </c>
+      <c r="O71">
+        <v>1</v>
+      </c>
+      <c r="P71" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>825</v>
+      </c>
+      <c r="R71" t="s">
+        <v>825</v>
+      </c>
+      <c r="S71" t="s">
+        <v>826</v>
+      </c>
+      <c r="T71" t="s">
+        <v>825</v>
+      </c>
+      <c r="U71" t="s">
+        <v>827</v>
+      </c>
+      <c r="V71" t="s">
+        <v>820</v>
+      </c>
+      <c r="W71" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B72" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C72" t="s">
+        <v>64</v>
+      </c>
+      <c r="D72" t="s">
+        <v>613</v>
+      </c>
+      <c r="E72" t="s">
+        <v>188</v>
+      </c>
+      <c r="F72" t="s">
+        <v>64</v>
+      </c>
+      <c r="G72" t="s">
+        <v>60</v>
+      </c>
+      <c r="H72" t="s">
+        <v>818</v>
+      </c>
+      <c r="I72" t="s">
+        <v>819</v>
+      </c>
+      <c r="J72" t="s">
+        <v>820</v>
+      </c>
+      <c r="K72" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L72" t="s">
+        <v>1101</v>
+      </c>
+      <c r="M72" t="s">
+        <v>1102</v>
+      </c>
+      <c r="N72">
+        <v>1906</v>
+      </c>
+      <c r="O72">
+        <v>1</v>
+      </c>
+      <c r="P72" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>825</v>
+      </c>
+      <c r="R72" t="s">
+        <v>825</v>
+      </c>
+      <c r="S72" t="s">
+        <v>826</v>
+      </c>
+      <c r="T72" t="s">
+        <v>825</v>
+      </c>
+      <c r="U72" t="s">
+        <v>827</v>
+      </c>
+      <c r="V72" t="s">
+        <v>820</v>
+      </c>
+      <c r="W72" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B73" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C73" t="s">
+        <v>64</v>
+      </c>
+      <c r="D73" t="s">
+        <v>56</v>
+      </c>
+      <c r="E73" t="s">
+        <v>61</v>
+      </c>
+      <c r="F73" t="s">
+        <v>64</v>
+      </c>
+      <c r="G73" t="s">
+        <v>60</v>
+      </c>
+      <c r="H73" t="s">
+        <v>818</v>
+      </c>
+      <c r="I73" t="s">
+        <v>819</v>
+      </c>
+      <c r="J73" t="s">
+        <v>820</v>
+      </c>
+      <c r="K73" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L73" t="s">
+        <v>1105</v>
+      </c>
+      <c r="M73" t="s">
+        <v>1106</v>
+      </c>
+      <c r="N73">
+        <v>2053</v>
+      </c>
+      <c r="O73">
+        <v>1</v>
+      </c>
+      <c r="P73" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>825</v>
+      </c>
+      <c r="R73" t="s">
+        <v>825</v>
+      </c>
+      <c r="S73" t="s">
+        <v>826</v>
+      </c>
+      <c r="T73" t="s">
+        <v>825</v>
+      </c>
+      <c r="U73" t="s">
+        <v>827</v>
+      </c>
+      <c r="V73" t="s">
+        <v>820</v>
+      </c>
+      <c r="W73" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B74" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C74" t="s">
+        <v>64</v>
+      </c>
+      <c r="D74" t="s">
+        <v>427</v>
+      </c>
+      <c r="E74" t="s">
+        <v>34</v>
+      </c>
+      <c r="F74" t="s">
+        <v>64</v>
+      </c>
+      <c r="G74" t="s">
+        <v>60</v>
+      </c>
+      <c r="H74" t="s">
+        <v>818</v>
+      </c>
+      <c r="I74" t="s">
+        <v>819</v>
+      </c>
+      <c r="J74" t="s">
+        <v>820</v>
+      </c>
+      <c r="K74" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L74" t="s">
+        <v>1108</v>
+      </c>
+      <c r="M74" t="s">
+        <v>1109</v>
+      </c>
+      <c r="N74">
+        <v>2402</v>
+      </c>
+      <c r="O74">
+        <v>1</v>
+      </c>
+      <c r="P74" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q74" t="s">
+        <v>825</v>
+      </c>
+      <c r="R74" t="s">
+        <v>825</v>
+      </c>
+      <c r="S74" t="s">
+        <v>826</v>
+      </c>
+      <c r="T74" t="s">
+        <v>825</v>
+      </c>
+      <c r="U74" t="s">
+        <v>827</v>
+      </c>
+      <c r="V74" t="s">
+        <v>820</v>
+      </c>
+      <c r="W74" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B75" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C75" t="s">
+        <v>64</v>
+      </c>
+      <c r="D75" t="s">
+        <v>613</v>
+      </c>
+      <c r="E75" t="s">
+        <v>188</v>
+      </c>
+      <c r="F75" t="s">
+        <v>64</v>
+      </c>
+      <c r="G75" t="s">
+        <v>60</v>
+      </c>
+      <c r="H75" t="s">
+        <v>818</v>
+      </c>
+      <c r="I75" t="s">
+        <v>819</v>
+      </c>
+      <c r="J75" t="s">
+        <v>820</v>
+      </c>
+      <c r="K75" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L75" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M75" t="s">
+        <v>1112</v>
+      </c>
+      <c r="N75">
+        <v>2374</v>
+      </c>
+      <c r="O75">
+        <v>1</v>
+      </c>
+      <c r="P75" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>825</v>
+      </c>
+      <c r="R75" t="s">
+        <v>825</v>
+      </c>
+      <c r="S75" t="s">
+        <v>826</v>
+      </c>
+      <c r="T75" t="s">
+        <v>825</v>
+      </c>
+      <c r="U75" t="s">
+        <v>827</v>
+      </c>
+      <c r="V75" t="s">
+        <v>820</v>
+      </c>
+      <c r="W75" t="s">
+        <v>825</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>